<commit_message>
Publish post-repair tables, candidate export and checked slides
The independent global review passes 29,129 checks with zero discrepancies and stable inputs, rechecked before publication. The refreshed candidate export passes 565 arithmetic checks and includes native potentials for 34 original proposals plus 22/25 complete additional pairs. Record 395 passing software tests and keep the three remaining new candidates, spin-ensemble integration, solution kinetics and exact-graft accuracy explicit. Preserve pre-existing staged archive changes.
</commit_message>
<xml_diff>
--- a/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
+++ b/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
@@ -3405,7 +3405,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>partial native solution states; remaining states pending</t>
+          <t>native solution states complete</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -3496,23 +3496,31 @@
         <v>3</v>
       </c>
       <c r="AD8" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF8" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AG8" s="2" t="n"/>
-      <c r="AH8" s="2" t="n"/>
-      <c r="AI8" s="2" t="n"/>
-      <c r="AJ8" s="2" t="n"/>
-      <c r="AK8" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+        <v>3</v>
+      </c>
+      <c r="AF8" s="2" t="inlineStr">
+        <is>
+          <t>verified native calculation</t>
+        </is>
+      </c>
+      <c r="AG8" s="3" t="n">
+        <v>-0.7458622613339685</v>
+      </c>
+      <c r="AH8" s="3" t="n">
+        <v>-1.420937286049593</v>
+      </c>
+      <c r="AI8" s="3" t="n">
+        <v>0.6750750247156247</v>
+      </c>
+      <c r="AJ8" s="3" t="n">
+        <v>65.13483796560426</v>
+      </c>
+      <c r="AK8" s="2" t="inlineStr">
+        <is>
+          <t>native thermodynamic calculation; decomposition untested</t>
         </is>
       </c>
       <c r="AL8" s="4" t="inlineStr">
@@ -3524,10 +3532,12 @@
       <c r="AN8" s="2" t="n"/>
       <c r="AO8" s="2" t="inlineStr">
         <is>
-          <t>pending electrolyte-window/integrity QC</t>
-        </is>
-      </c>
-      <c r="AP8" s="2" t="n"/>
+          <t>computed native-window/integrity bookkeeping; kinetic QC separate</t>
+        </is>
+      </c>
+      <c r="AP8" s="3" t="n">
+        <v>125.1107782788156</v>
+      </c>
       <c r="AQ8" s="2" t="b">
         <v>0</v>
       </c>
@@ -3546,7 +3556,7 @@
       </c>
       <c r="AU8" s="2" t="inlineStr">
         <is>
-          <t>native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV8" s="2" t="n"/>
@@ -3556,7 +3566,7 @@
       <c r="AZ8" s="2" t="n"/>
       <c r="BA8" s="2" t="n"/>
       <c r="BB8" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC8" s="2" t="inlineStr">
         <is>
@@ -3568,8 +3578,12 @@
           <t>neu:UMA_large_gap_preliminary; red1:standard_doublet_model; red2:UMA_large_gap_preliminary</t>
         </is>
       </c>
-      <c r="BE8" s="2" t="n"/>
-      <c r="BF8" s="2" t="n"/>
+      <c r="BE8" s="3" t="n">
+        <v>-0.7458622613339685</v>
+      </c>
+      <c r="BF8" s="3" t="n">
+        <v>-1.420937286049593</v>
+      </c>
       <c r="BG8" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
@@ -7653,7 +7667,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>partial native solution states; remaining states pending</t>
+          <t>native solution states complete</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -7744,23 +7758,31 @@
         <v>3</v>
       </c>
       <c r="AD28" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE28" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF28" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AG28" s="2" t="n"/>
-      <c r="AH28" s="2" t="n"/>
-      <c r="AI28" s="2" t="n"/>
-      <c r="AJ28" s="2" t="n"/>
-      <c r="AK28" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+        <v>3</v>
+      </c>
+      <c r="AF28" s="2" t="inlineStr">
+        <is>
+          <t>verified native calculation</t>
+        </is>
+      </c>
+      <c r="AG28" s="3" t="n">
+        <v>-0.7561418107361533</v>
+      </c>
+      <c r="AH28" s="3" t="n">
+        <v>-1.414662151400989</v>
+      </c>
+      <c r="AI28" s="3" t="n">
+        <v>0.6585203406721121</v>
+      </c>
+      <c r="AJ28" s="3" t="n">
+        <v>63.53755377752429</v>
+      </c>
+      <c r="AK28" s="2" t="inlineStr">
+        <is>
+          <t>native thermodynamic calculation; decomposition untested</t>
         </is>
       </c>
       <c r="AL28" s="4" t="inlineStr">
@@ -7772,10 +7794,12 @@
       <c r="AN28" s="2" t="n"/>
       <c r="AO28" s="2" t="inlineStr">
         <is>
-          <t>pending electrolyte-window/integrity QC</t>
-        </is>
-      </c>
-      <c r="AP28" s="2" t="n"/>
+          <t>computed native-window/integrity bookkeeping; kinetic QC separate</t>
+        </is>
+      </c>
+      <c r="AP28" s="3" t="n">
+        <v>125.6892886025082</v>
+      </c>
       <c r="AQ28" s="2" t="b">
         <v>0</v>
       </c>
@@ -7794,7 +7818,7 @@
       </c>
       <c r="AU28" s="2" t="inlineStr">
         <is>
-          <t>native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV28" s="2" t="n"/>
@@ -7804,7 +7828,7 @@
       <c r="AZ28" s="2" t="n"/>
       <c r="BA28" s="2" t="n"/>
       <c r="BB28" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC28" s="2" t="inlineStr">
         <is>
@@ -7816,8 +7840,12 @@
           <t>neu:UMA_large_gap_preliminary; red1:standard_doublet_model; red2:UMA_large_gap_preliminary</t>
         </is>
       </c>
-      <c r="BE28" s="2" t="n"/>
-      <c r="BF28" s="2" t="n"/>
+      <c r="BE28" s="3" t="n">
+        <v>-0.7561418107361533</v>
+      </c>
+      <c r="BF28" s="3" t="n">
+        <v>-1.414662151400989</v>
+      </c>
       <c r="BG28" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
@@ -13205,14 +13233,16 @@
         </is>
       </c>
       <c r="R21" s="3" t="n">
-        <v>-39474.39661079711</v>
-      </c>
-      <c r="S21" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T21" s="2" t="n"/>
+        <v>-39474.39858469691</v>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T21" s="3" t="n">
+        <v>9.433571384692929</v>
+      </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
           <t>native_solution_dft_qrrho_spin</t>
@@ -13220,18 +13250,16 @@
       </c>
       <c r="V21" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="W21" s="2" t="inlineStr">
-        <is>
-          <t>missing_validated_native_thermal</t>
-        </is>
-      </c>
-      <c r="X21" s="2" t="n"/>
-      <c r="Y21" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr"/>
+      <c r="X21" s="3" t="n">
+        <v>-39464.96501331221</v>
+      </c>
+      <c r="Y21" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
         </is>
       </c>
       <c r="Z21" s="2" t="inlineStr">
@@ -13263,7 +13291,9 @@
       <c r="AF21" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AG21" s="2" t="n"/>
+      <c r="AG21" s="3" t="n">
+        <v>-39464.96501331221</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -21131,14 +21161,16 @@
         </is>
       </c>
       <c r="R81" s="3" t="n">
-        <v>-38497.07854302814</v>
-      </c>
-      <c r="S81" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T81" s="2" t="n"/>
+        <v>-38497.12193000768</v>
+      </c>
+      <c r="S81" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T81" s="3" t="n">
+        <v>10.06697745373095</v>
+      </c>
       <c r="U81" s="2" t="inlineStr">
         <is>
           <t>native_solution_dft_qrrho_spin</t>
@@ -21146,18 +21178,16 @@
       </c>
       <c r="V81" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="W81" s="2" t="inlineStr">
-        <is>
-          <t>missing_validated_native_thermal</t>
-        </is>
-      </c>
-      <c r="X81" s="2" t="n"/>
-      <c r="Y81" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="W81" s="2" t="inlineStr"/>
+      <c r="X81" s="3" t="n">
+        <v>-38487.05495255395</v>
+      </c>
+      <c r="Y81" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
         </is>
       </c>
       <c r="Z81" s="2" t="inlineStr">
@@ -21189,7 +21219,9 @@
       <c r="AF81" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AG81" s="2" t="n"/>
+      <c r="AG81" s="3" t="n">
+        <v>-38487.05495255395</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -37189,10 +37221,12 @@
       <c r="F14" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="G14" s="3" t="n">
+        <v>-0.7458622613339685</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -37201,7 +37235,7 @@
         </is>
       </c>
       <c r="J14" s="3" t="n">
-        <v>3.542</v>
+        <v>3.544</v>
       </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
@@ -37228,7 +37262,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="R14" s="2" t="n"/>
+      <c r="R14" s="3" t="n">
+        <v>-0.7458622613339685</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -37257,10 +37293,12 @@
       <c r="F15" s="2" t="n">
         <v>-2</v>
       </c>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="G15" s="3" t="n">
+        <v>-1.420937286049593</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -37269,7 +37307,7 @@
         </is>
       </c>
       <c r="J15" s="3" t="n">
-        <v>2.932</v>
+        <v>2.93</v>
       </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n"/>
@@ -37296,7 +37334,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="R15" s="2" t="n"/>
+      <c r="R15" s="3" t="n">
+        <v>-1.420937286049593</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -40127,10 +40167,12 @@
       <c r="F54" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="G54" s="2" t="n"/>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="G54" s="3" t="n">
+        <v>-0.7561418107361533</v>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -40139,7 +40181,7 @@
         </is>
       </c>
       <c r="J54" s="3" t="n">
-        <v>3.5</v>
+        <v>3.543</v>
       </c>
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="n"/>
@@ -40166,7 +40208,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="R54" s="2" t="n"/>
+      <c r="R54" s="3" t="n">
+        <v>-0.7561418107361533</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -40195,10 +40239,12 @@
       <c r="F55" s="2" t="n">
         <v>-2</v>
       </c>
-      <c r="G55" s="2" t="n"/>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="G55" s="3" t="n">
+        <v>-1.414662151400989</v>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -40207,7 +40253,7 @@
         </is>
       </c>
       <c r="J55" s="3" t="n">
-        <v>2.982</v>
+        <v>2.939</v>
       </c>
       <c r="K55" s="2" t="n"/>
       <c r="L55" s="2" t="n"/>
@@ -40234,7 +40280,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="R55" s="2" t="n"/>
+      <c r="R55" s="3" t="n">
+        <v>-1.414662151400989</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -53230,7 +53278,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-19T00:21:03.626186-05:00</t>
+          <t>2026-10-19T00:38:00.450031-05:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish model-qualified candidate exports and checked force diagnostics
</commit_message>
<xml_diff>
--- a/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
+++ b/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
@@ -16,11 +16,11 @@
     <sheet name="Conventions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Original39'!$A$1:$BH$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Original39'!$A$1:$BM$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'States'!$A$1:$AL$194</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Couples'!$A$1:$T$129</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Additional'!$A$1:$BH$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Controls'!$A$1:$BH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Additional'!$A$1:$BM$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Controls'!$A$1:$BM$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Comparisons'!$A$1:$I$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -378,7 +378,7 @@
     </comment>
     <comment ref="AP1" authorId="0" shapeId="0">
       <text>
-        <t>Native potential window and integrity-contiguous path bookkeeping; kinetics assessed separately.</t>
+        <t>Native potential window and integrity-contiguous path bookkeeping, withheld where a scoped model limitation applies; kinetics assessed separately.</t>
       </text>
     </comment>
     <comment ref="AQ1" authorId="0" shapeId="0">
@@ -467,6 +467,31 @@
       </text>
     </comment>
     <comment ref="BH1" authorId="0" shapeId="0">
+      <text>
+        <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
+      </text>
+    </comment>
+    <comment ref="BI1" authorId="0" shapeId="0">
+      <text>
+        <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
+      </text>
+    </comment>
+    <comment ref="BJ1" authorId="0" shapeId="0">
+      <text>
+        <t>Largest reviewed free-parent residual for the scoped model limitation; never a measurement or error bound for an exact graft.</t>
+      </text>
+    </comment>
+    <comment ref="BK1" authorId="0" shapeId="0">
+      <text>
+        <t>Original model window/path estimate retained for diagnosis; not qualified capacity when model_primary_admissible is false.</t>
+      </text>
+    </comment>
+    <comment ref="BL1" authorId="0" shapeId="0">
+      <text>
+        <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
+      </text>
+    </comment>
+    <comment ref="BM1" authorId="0" shapeId="0">
       <text>
         <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
       </text>
@@ -998,7 +1023,7 @@
     </comment>
     <comment ref="AP1" authorId="0" shapeId="0">
       <text>
-        <t>Native potential window and integrity-contiguous path bookkeeping; kinetics assessed separately.</t>
+        <t>Native potential window and integrity-contiguous path bookkeeping, withheld where a scoped model limitation applies; kinetics assessed separately.</t>
       </text>
     </comment>
     <comment ref="AQ1" authorId="0" shapeId="0">
@@ -1087,6 +1112,31 @@
       </text>
     </comment>
     <comment ref="BH1" authorId="0" shapeId="0">
+      <text>
+        <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
+      </text>
+    </comment>
+    <comment ref="BI1" authorId="0" shapeId="0">
+      <text>
+        <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
+      </text>
+    </comment>
+    <comment ref="BJ1" authorId="0" shapeId="0">
+      <text>
+        <t>Largest reviewed free-parent residual for the scoped model limitation; never a measurement or error bound for an exact graft.</t>
+      </text>
+    </comment>
+    <comment ref="BK1" authorId="0" shapeId="0">
+      <text>
+        <t>Original model window/path estimate retained for diagnosis; not qualified capacity when model_primary_admissible is false.</t>
+      </text>
+    </comment>
+    <comment ref="BL1" authorId="0" shapeId="0">
+      <text>
+        <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
+      </text>
+    </comment>
+    <comment ref="BM1" authorId="0" shapeId="0">
       <text>
         <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
       </text>
@@ -1308,7 +1358,7 @@
     </comment>
     <comment ref="AP1" authorId="0" shapeId="0">
       <text>
-        <t>Native potential window and integrity-contiguous path bookkeeping; kinetics assessed separately.</t>
+        <t>Native potential window and integrity-contiguous path bookkeeping, withheld where a scoped model limitation applies; kinetics assessed separately.</t>
       </text>
     </comment>
     <comment ref="AQ1" authorId="0" shapeId="0">
@@ -1397,6 +1447,31 @@
       </text>
     </comment>
     <comment ref="BH1" authorId="0" shapeId="0">
+      <text>
+        <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
+      </text>
+    </comment>
+    <comment ref="BI1" authorId="0" shapeId="0">
+      <text>
+        <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
+      </text>
+    </comment>
+    <comment ref="BJ1" authorId="0" shapeId="0">
+      <text>
+        <t>Largest reviewed free-parent residual for the scoped model limitation; never a measurement or error bound for an exact graft.</t>
+      </text>
+    </comment>
+    <comment ref="BK1" authorId="0" shapeId="0">
+      <text>
+        <t>Original model window/path estimate retained for diagnosis; not qualified capacity when model_primary_admissible is false.</t>
+      </text>
+    </comment>
+    <comment ref="BL1" authorId="0" shapeId="0">
+      <text>
+        <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
+      </text>
+    </comment>
+    <comment ref="BM1" authorId="0" shapeId="0">
       <text>
         <t>Snapshot exported from exact-structure pipeline records; blank means not computed/validated.</t>
       </text>
@@ -1749,7 +1824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH40"/>
+  <dimension ref="A1:BM40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1811,7 +1886,12 @@
     <col width="22" customWidth="1" min="57" max="57"/>
     <col width="22" customWidth="1" min="58" max="58"/>
     <col width="22" customWidth="1" min="59" max="59"/>
-    <col width="22" customWidth="1" min="60" max="60"/>
+    <col width="35" customWidth="1" min="60" max="60"/>
+    <col width="22" customWidth="1" min="61" max="61"/>
+    <col width="22" customWidth="1" min="62" max="62"/>
+    <col width="22" customWidth="1" min="63" max="63"/>
+    <col width="22" customWidth="1" min="64" max="64"/>
+    <col width="22" customWidth="1" min="65" max="65"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -2107,10 +2187,35 @@
       </c>
       <c r="BG1" s="1" t="inlineStr">
         <is>
+          <t>model_primary_admissible</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>model_validation_status</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>model_validation_evidence</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>model_max_observed_error_V</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>model_accessible_capacity_estimate_mAh_g</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
           <t>fleet_progress</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
         <is>
           <t>experimentally_validated_for_exact_graft</t>
         </is>
@@ -2323,12 +2428,25 @@
       <c r="BF2" s="3" t="n">
         <v>-1.976641698471212</v>
       </c>
-      <c r="BG2" s="2" t="inlineStr">
+      <c r="BG2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH2" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI2" s="2" t="n"/>
+      <c r="BJ2" s="2" t="n"/>
+      <c r="BK2" s="3" t="n">
+        <v>153.8732059803102</v>
+      </c>
+      <c r="BL2" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH2" s="2" t="b">
+      <c r="BM2" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2539,12 +2657,25 @@
       <c r="BF3" s="3" t="n">
         <v>-1.948399842643994</v>
       </c>
-      <c r="BG3" s="2" t="inlineStr">
+      <c r="BG3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH3" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI3" s="2" t="n"/>
+      <c r="BJ3" s="2" t="n"/>
+      <c r="BK3" s="3" t="n">
+        <v>141.6628670580386</v>
+      </c>
+      <c r="BL3" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH3" s="2" t="b">
+      <c r="BM3" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2755,12 +2886,25 @@
       <c r="BF4" s="3" t="n">
         <v>-1.967852708316059</v>
       </c>
-      <c r="BG4" s="2" t="inlineStr">
+      <c r="BG4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH4" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI4" s="2" t="n"/>
+      <c r="BJ4" s="2" t="n"/>
+      <c r="BK4" s="3" t="n">
+        <v>126.8898375116027</v>
+      </c>
+      <c r="BL4" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH4" s="2" t="b">
+      <c r="BM4" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2971,12 +3115,25 @@
       <c r="BF5" s="3" t="n">
         <v>-1.980917624583526</v>
       </c>
-      <c r="BG5" s="2" t="inlineStr">
+      <c r="BG5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH5" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI5" s="2" t="n"/>
+      <c r="BJ5" s="2" t="n"/>
+      <c r="BK5" s="3" t="n">
+        <v>147.9171662427774</v>
+      </c>
+      <c r="BL5" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH5" s="2" t="b">
+      <c r="BM5" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3187,12 +3344,25 @@
       <c r="BF6" s="3" t="n">
         <v>-1.399670212304045</v>
       </c>
-      <c r="BG6" s="2" t="inlineStr">
+      <c r="BG6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH6" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI6" s="2" t="n"/>
+      <c r="BJ6" s="2" t="n"/>
+      <c r="BK6" s="3" t="n">
+        <v>139.4490565306911</v>
+      </c>
+      <c r="BL6" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH6" s="2" t="b">
+      <c r="BM6" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3403,12 +3573,25 @@
       <c r="BF7" s="3" t="n">
         <v>-1.418482689237862</v>
       </c>
-      <c r="BG7" s="2" t="inlineStr">
+      <c r="BG7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH7" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI7" s="2" t="n"/>
+      <c r="BJ7" s="2" t="n"/>
+      <c r="BK7" s="3" t="n">
+        <v>134.5395094822244</v>
+      </c>
+      <c r="BL7" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH7" s="2" t="b">
+      <c r="BM7" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3619,12 +3802,25 @@
       <c r="BF8" s="3" t="n">
         <v>-1.420937286049593</v>
       </c>
-      <c r="BG8" s="2" t="inlineStr">
+      <c r="BG8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH8" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI8" s="2" t="n"/>
+      <c r="BJ8" s="2" t="n"/>
+      <c r="BK8" s="3" t="n">
+        <v>125.1107782788156</v>
+      </c>
+      <c r="BL8" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH8" s="2" t="b">
+      <c r="BM8" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3825,12 +4021,23 @@
         <v>-0.8081823078682646</v>
       </c>
       <c r="BF9" s="2" t="n"/>
-      <c r="BG9" s="2" t="inlineStr">
+      <c r="BG9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH9" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI9" s="2" t="n"/>
+      <c r="BJ9" s="2" t="n"/>
+      <c r="BK9" s="2" t="n"/>
+      <c r="BL9" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH9" s="2" t="b">
+      <c r="BM9" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4041,12 +4248,25 @@
       <c r="BF10" s="3" t="n">
         <v>-1.415987651278556</v>
       </c>
-      <c r="BG10" s="2" t="inlineStr">
+      <c r="BG10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH10" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI10" s="2" t="n"/>
+      <c r="BJ10" s="2" t="n"/>
+      <c r="BK10" s="3" t="n">
+        <v>129.9639037662934</v>
+      </c>
+      <c r="BL10" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH10" s="2" t="b">
+      <c r="BM10" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4243,12 +4463,23 @@
       </c>
       <c r="BE11" s="2" t="n"/>
       <c r="BF11" s="2" t="n"/>
-      <c r="BG11" s="2" t="inlineStr">
+      <c r="BG11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH11" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI11" s="2" t="n"/>
+      <c r="BJ11" s="2" t="n"/>
+      <c r="BK11" s="2" t="n"/>
+      <c r="BL11" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH11" s="2" t="b">
+      <c r="BM11" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4449,12 +4680,23 @@
       <c r="BF12" s="3" t="n">
         <v>-1.713479404512327</v>
       </c>
-      <c r="BG12" s="2" t="inlineStr">
+      <c r="BG12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH12" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI12" s="2" t="n"/>
+      <c r="BJ12" s="2" t="n"/>
+      <c r="BK12" s="2" t="n"/>
+      <c r="BL12" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH12" s="2" t="b">
+      <c r="BM12" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4665,12 +4907,25 @@
       <c r="BF13" s="3" t="n">
         <v>-1.785621345130494</v>
       </c>
-      <c r="BG13" s="2" t="inlineStr">
+      <c r="BG13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH13" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI13" s="2" t="n"/>
+      <c r="BJ13" s="2" t="n"/>
+      <c r="BK13" s="3" t="n">
+        <v>150.4775497345422</v>
+      </c>
+      <c r="BL13" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH13" s="2" t="b">
+      <c r="BM13" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4881,12 +5136,25 @@
       <c r="BF14" s="3" t="n">
         <v>-1.800414359109709</v>
       </c>
-      <c r="BG14" s="2" t="inlineStr">
+      <c r="BG14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH14" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI14" s="2" t="n"/>
+      <c r="BJ14" s="2" t="n"/>
+      <c r="BK14" s="3" t="n">
+        <v>171.9322133409744</v>
+      </c>
+      <c r="BL14" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH14" s="2" t="b">
+      <c r="BM14" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5097,12 +5365,25 @@
       <c r="BF15" s="3" t="n">
         <v>-1.312758876738371</v>
       </c>
-      <c r="BG15" s="2" t="inlineStr">
+      <c r="BG15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH15" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI15" s="2" t="n"/>
+      <c r="BJ15" s="2" t="n"/>
+      <c r="BK15" s="3" t="n">
+        <v>73.79343699942852</v>
+      </c>
+      <c r="BL15" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH15" s="2" t="b">
+      <c r="BM15" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5313,12 +5594,25 @@
       <c r="BF16" s="3" t="n">
         <v>-1.895350608629087</v>
       </c>
-      <c r="BG16" s="2" t="inlineStr">
+      <c r="BG16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH16" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI16" s="2" t="n"/>
+      <c r="BJ16" s="2" t="n"/>
+      <c r="BK16" s="3" t="n">
+        <v>183.3595437092984</v>
+      </c>
+      <c r="BL16" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH16" s="2" t="b">
+      <c r="BM16" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5529,12 +5823,25 @@
       <c r="BF17" s="3" t="n">
         <v>-1.566273036383791</v>
       </c>
-      <c r="BG17" s="2" t="inlineStr">
+      <c r="BG17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH17" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI17" s="2" t="n"/>
+      <c r="BJ17" s="2" t="n"/>
+      <c r="BK17" s="3" t="n">
+        <v>164.0322853051991</v>
+      </c>
+      <c r="BL17" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH17" s="2" t="b">
+      <c r="BM17" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5745,12 +6052,25 @@
       <c r="BF18" s="3" t="n">
         <v>-1.999523098573263</v>
       </c>
-      <c r="BG18" s="2" t="inlineStr">
+      <c r="BG18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH18" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI18" s="2" t="n"/>
+      <c r="BJ18" s="2" t="n"/>
+      <c r="BK18" s="3" t="n">
+        <v>166.79205133205</v>
+      </c>
+      <c r="BL18" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH18" s="2" t="b">
+      <c r="BM18" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5961,12 +6281,25 @@
       <c r="BF19" s="3" t="n">
         <v>-1.849600849400304</v>
       </c>
-      <c r="BG19" s="2" t="inlineStr">
+      <c r="BG19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH19" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI19" s="2" t="n"/>
+      <c r="BJ19" s="2" t="n"/>
+      <c r="BK19" s="3" t="n">
+        <v>160.7617836640531</v>
+      </c>
+      <c r="BL19" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH19" s="2" t="b">
+      <c r="BM19" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6177,12 +6510,25 @@
       <c r="BF20" s="3" t="n">
         <v>-1.888461510359775</v>
       </c>
-      <c r="BG20" s="2" t="inlineStr">
+      <c r="BG20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH20" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI20" s="2" t="n"/>
+      <c r="BJ20" s="2" t="n"/>
+      <c r="BK20" s="3" t="n">
+        <v>154.7313489428879</v>
+      </c>
+      <c r="BL20" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH20" s="2" t="b">
+      <c r="BM20" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6383,12 +6729,23 @@
       <c r="BF21" s="3" t="n">
         <v>-1.881490726009361</v>
       </c>
-      <c r="BG21" s="2" t="inlineStr">
+      <c r="BG21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH21" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI21" s="2" t="n"/>
+      <c r="BJ21" s="2" t="n"/>
+      <c r="BK21" s="2" t="n"/>
+      <c r="BL21" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH21" s="2" t="b">
+      <c r="BM21" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6599,12 +6956,25 @@
       <c r="BF22" s="3" t="n">
         <v>-1.908879687623994</v>
       </c>
-      <c r="BG22" s="2" t="inlineStr">
+      <c r="BG22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH22" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI22" s="2" t="n"/>
+      <c r="BJ22" s="2" t="n"/>
+      <c r="BK22" s="3" t="n">
+        <v>161.2609011726536</v>
+      </c>
+      <c r="BL22" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH22" s="2" t="b">
+      <c r="BM22" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6815,12 +7185,25 @@
       <c r="BF23" s="3" t="n">
         <v>-1.9260421876279</v>
       </c>
-      <c r="BG23" s="2" t="inlineStr">
+      <c r="BG23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH23" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI23" s="2" t="n"/>
+      <c r="BJ23" s="2" t="n"/>
+      <c r="BK23" s="3" t="n">
+        <v>167.3063981450269</v>
+      </c>
+      <c r="BL23" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH23" s="2" t="b">
+      <c r="BM23" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7031,12 +7414,25 @@
       <c r="BF24" s="3" t="n">
         <v>-2.00566952189547</v>
       </c>
-      <c r="BG24" s="2" t="inlineStr">
+      <c r="BG24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH24" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI24" s="2" t="n"/>
+      <c r="BJ24" s="2" t="n"/>
+      <c r="BK24" s="3" t="n">
+        <v>153.836111286495</v>
+      </c>
+      <c r="BL24" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH24" s="2" t="b">
+      <c r="BM24" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7247,12 +7643,25 @@
       <c r="BF25" s="3" t="n">
         <v>-1.963524694561784</v>
       </c>
-      <c r="BG25" s="2" t="inlineStr">
+      <c r="BG25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH25" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI25" s="2" t="n"/>
+      <c r="BJ25" s="2" t="n"/>
+      <c r="BK25" s="3" t="n">
+        <v>172.7183341621494</v>
+      </c>
+      <c r="BL25" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH25" s="2" t="b">
+      <c r="BM25" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7463,12 +7872,25 @@
       <c r="BF26" s="3" t="n">
         <v>-1.980617244633322</v>
       </c>
-      <c r="BG26" s="2" t="inlineStr">
+      <c r="BG26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH26" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI26" s="2" t="n"/>
+      <c r="BJ26" s="2" t="n"/>
+      <c r="BK26" s="3" t="n">
+        <v>142.4050303627113</v>
+      </c>
+      <c r="BL26" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH26" s="2" t="b">
+      <c r="BM26" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7665,12 +8087,23 @@
       </c>
       <c r="BE27" s="2" t="n"/>
       <c r="BF27" s="2" t="n"/>
-      <c r="BG27" s="2" t="inlineStr">
+      <c r="BG27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH27" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI27" s="2" t="n"/>
+      <c r="BJ27" s="2" t="n"/>
+      <c r="BK27" s="2" t="n"/>
+      <c r="BL27" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH27" s="2" t="b">
+      <c r="BM27" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7881,12 +8314,25 @@
       <c r="BF28" s="3" t="n">
         <v>-1.414662151400989</v>
       </c>
-      <c r="BG28" s="2" t="inlineStr">
+      <c r="BG28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH28" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI28" s="2" t="n"/>
+      <c r="BJ28" s="2" t="n"/>
+      <c r="BK28" s="3" t="n">
+        <v>125.6892886025082</v>
+      </c>
+      <c r="BL28" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH28" s="2" t="b">
+      <c r="BM28" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8097,12 +8543,25 @@
       <c r="BF29" s="3" t="n">
         <v>-1.326003791175026</v>
       </c>
-      <c r="BG29" s="2" t="inlineStr">
+      <c r="BG29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH29" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI29" s="2" t="n"/>
+      <c r="BJ29" s="2" t="n"/>
+      <c r="BK29" s="3" t="n">
+        <v>103.7711011303628</v>
+      </c>
+      <c r="BL29" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH29" s="2" t="b">
+      <c r="BM29" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8313,12 +8772,25 @@
       <c r="BF30" s="3" t="n">
         <v>-1.966158162380452</v>
       </c>
-      <c r="BG30" s="2" t="inlineStr">
+      <c r="BG30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH30" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI30" s="2" t="n"/>
+      <c r="BJ30" s="2" t="n"/>
+      <c r="BK30" s="3" t="n">
+        <v>137.2889549683533</v>
+      </c>
+      <c r="BL30" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH30" s="2" t="b">
+      <c r="BM30" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8529,12 +9001,25 @@
       <c r="BF31" s="3" t="n">
         <v>-1.976572419858712</v>
       </c>
-      <c r="BG31" s="2" t="inlineStr">
+      <c r="BG31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH31" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI31" s="2" t="n"/>
+      <c r="BJ31" s="2" t="n"/>
+      <c r="BK31" s="3" t="n">
+        <v>137.2889549683533</v>
+      </c>
+      <c r="BL31" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH31" s="2" t="b">
+      <c r="BM31" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8745,12 +9230,25 @@
       <c r="BF32" s="3" t="n">
         <v>-2.016746385088481</v>
       </c>
-      <c r="BG32" s="2" t="inlineStr">
+      <c r="BG32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH32" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI32" s="2" t="n"/>
+      <c r="BJ32" s="2" t="n"/>
+      <c r="BK32" s="3" t="n">
+        <v>163.2410147453577</v>
+      </c>
+      <c r="BL32" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH32" s="2" t="b">
+      <c r="BM32" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8961,12 +9459,25 @@
       <c r="BF33" s="3" t="n">
         <v>-2.082040487006452</v>
       </c>
-      <c r="BG33" s="2" t="inlineStr">
+      <c r="BG33" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH33" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI33" s="2" t="n"/>
+      <c r="BJ33" s="2" t="n"/>
+      <c r="BK33" s="3" t="n">
+        <v>149.5647579302299</v>
+      </c>
+      <c r="BL33" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH33" s="2" t="b">
+      <c r="BM33" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -9177,12 +9688,25 @@
       <c r="BF34" s="3" t="n">
         <v>-1.765704975459812</v>
       </c>
-      <c r="BG34" s="2" t="inlineStr">
+      <c r="BG34" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH34" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI34" s="2" t="n"/>
+      <c r="BJ34" s="2" t="n"/>
+      <c r="BK34" s="3" t="n">
+        <v>207.5438094144138</v>
+      </c>
+      <c r="BL34" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH34" s="2" t="b">
+      <c r="BM34" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -9393,12 +9917,25 @@
       <c r="BF35" s="3" t="n">
         <v>-1.966520643396507</v>
       </c>
-      <c r="BG35" s="2" t="inlineStr">
+      <c r="BG35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH35" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI35" s="2" t="n"/>
+      <c r="BJ35" s="2" t="n"/>
+      <c r="BK35" s="3" t="n">
+        <v>198.2886060226425</v>
+      </c>
+      <c r="BL35" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH35" s="2" t="b">
+      <c r="BM35" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -9609,12 +10146,25 @@
       <c r="BF36" s="3" t="n">
         <v>-1.204313008285681</v>
       </c>
-      <c r="BG36" s="2" t="inlineStr">
+      <c r="BG36" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH36" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI36" s="2" t="n"/>
+      <c r="BJ36" s="2" t="n"/>
+      <c r="BK36" s="3" t="n">
+        <v>167.2813363320254</v>
+      </c>
+      <c r="BL36" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH36" s="2" t="b">
+      <c r="BM36" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -9825,12 +10375,25 @@
       <c r="BF37" s="3" t="n">
         <v>-1.150453106754867</v>
       </c>
-      <c r="BG37" s="2" t="inlineStr">
+      <c r="BG37" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH37" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI37" s="2" t="n"/>
+      <c r="BJ37" s="2" t="n"/>
+      <c r="BK37" s="3" t="n">
+        <v>147.0633195758689</v>
+      </c>
+      <c r="BL37" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH37" s="2" t="b">
+      <c r="BM37" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10033,12 +10596,25 @@
         <v>-1.641956213712547</v>
       </c>
       <c r="BF38" s="2" t="n"/>
-      <c r="BG38" s="2" t="inlineStr">
+      <c r="BG38" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH38" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI38" s="2" t="n"/>
+      <c r="BJ38" s="2" t="n"/>
+      <c r="BK38" s="3" t="n">
+        <v>106.6577039793241</v>
+      </c>
+      <c r="BL38" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH38" s="2" t="b">
+      <c r="BM38" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10241,12 +10817,25 @@
         <v>-1.521636358156684</v>
       </c>
       <c r="BF39" s="2" t="n"/>
-      <c r="BG39" s="2" t="inlineStr">
+      <c r="BG39" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH39" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI39" s="2" t="n"/>
+      <c r="BJ39" s="2" t="n"/>
+      <c r="BK39" s="3" t="n">
+        <v>88.93952494464631</v>
+      </c>
+      <c r="BL39" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH39" s="2" t="b">
+      <c r="BM39" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10405,12 +10994,10 @@
       <c r="AN40" s="2" t="n"/>
       <c r="AO40" s="2" t="inlineStr">
         <is>
-          <t>computed native-window/integrity bookkeeping; kinetic QC separate</t>
-        </is>
-      </c>
-      <c r="AP40" s="3" t="n">
-        <v>147.470747626812</v>
-      </c>
+          <t>provisional model window/path estimate; phenothiazine_second_oxidation_unqualified</t>
+        </is>
+      </c>
+      <c r="AP40" s="2" t="n"/>
       <c r="AQ40" s="2" t="b">
         <v>0</v>
       </c>
@@ -10457,17 +11044,36 @@
       <c r="BF40" s="3" t="n">
         <v>1.278506036345789</v>
       </c>
-      <c r="BG40" s="2" t="inlineStr">
+      <c r="BG40" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH40" s="2" t="inlineStr">
+        <is>
+          <t>phenothiazine_second_oxidation_unqualified</t>
+        </is>
+      </c>
+      <c r="BI40" s="2" t="inlineStr">
+        <is>
+          <t>results/reviews/2026-10-19/phenothiazine_checked_subset/model_discrepancy.json</t>
+        </is>
+      </c>
+      <c r="BJ40" s="3" t="n">
+        <v>0.547</v>
+      </c>
+      <c r="BK40" s="3" t="n">
+        <v>147.470747626812</v>
+      </c>
+      <c r="BL40" s="2" t="inlineStr">
         <is>
           <t>worker done marker; record QC separate</t>
         </is>
       </c>
-      <c r="BH40" s="2" t="b">
+      <c r="BM40" s="2" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BH40"/>
+  <autoFilter ref="A1:BM40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -48777,7 +49383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH26"/>
+  <dimension ref="A1:BM26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -48839,7 +49445,12 @@
     <col width="22" customWidth="1" min="57" max="57"/>
     <col width="22" customWidth="1" min="58" max="58"/>
     <col width="22" customWidth="1" min="59" max="59"/>
-    <col width="22" customWidth="1" min="60" max="60"/>
+    <col width="35" customWidth="1" min="60" max="60"/>
+    <col width="22" customWidth="1" min="61" max="61"/>
+    <col width="22" customWidth="1" min="62" max="62"/>
+    <col width="22" customWidth="1" min="63" max="63"/>
+    <col width="22" customWidth="1" min="64" max="64"/>
+    <col width="22" customWidth="1" min="65" max="65"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -49135,10 +49746,35 @@
       </c>
       <c r="BG1" s="1" t="inlineStr">
         <is>
+          <t>model_primary_admissible</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>model_validation_status</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>model_validation_evidence</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>model_max_observed_error_V</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>model_accessible_capacity_estimate_mAh_g</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
           <t>fleet_progress</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
         <is>
           <t>experimentally_validated_for_exact_graft</t>
         </is>
@@ -49333,12 +49969,23 @@
       </c>
       <c r="BE2" s="2" t="n"/>
       <c r="BF2" s="2" t="n"/>
-      <c r="BG2" s="2" t="inlineStr">
+      <c r="BG2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH2" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI2" s="2" t="n"/>
+      <c r="BJ2" s="2" t="n"/>
+      <c r="BK2" s="2" t="n"/>
+      <c r="BL2" s="2" t="inlineStr">
         <is>
           <t>terminal failure; partial data preserved</t>
         </is>
       </c>
-      <c r="BH2" s="2" t="b">
+      <c r="BM2" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -49545,12 +50192,25 @@
       <c r="BF3" s="3" t="n">
         <v>-1.962445311764895</v>
       </c>
-      <c r="BG3" s="2" t="inlineStr">
+      <c r="BG3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH3" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI3" s="2" t="n"/>
+      <c r="BJ3" s="2" t="n"/>
+      <c r="BK3" s="3" t="n">
+        <v>148.7446541985823</v>
+      </c>
+      <c r="BL3" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH3" s="2" t="b">
+      <c r="BM3" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -49757,12 +50417,25 @@
       <c r="BF4" s="3" t="n">
         <v>-1.937240352235676</v>
       </c>
-      <c r="BG4" s="2" t="inlineStr">
+      <c r="BG4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH4" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI4" s="2" t="n"/>
+      <c r="BJ4" s="2" t="n"/>
+      <c r="BK4" s="3" t="n">
+        <v>146.3170599781871</v>
+      </c>
+      <c r="BL4" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH4" s="2" t="b">
+      <c r="BM4" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -49969,12 +50642,25 @@
       <c r="BF5" s="3" t="n">
         <v>-1.394007067225175</v>
       </c>
-      <c r="BG5" s="2" t="inlineStr">
+      <c r="BG5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH5" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI5" s="2" t="n"/>
+      <c r="BJ5" s="2" t="n"/>
+      <c r="BK5" s="3" t="n">
+        <v>130.6022778334106</v>
+      </c>
+      <c r="BL5" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH5" s="2" t="b">
+      <c r="BM5" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -50181,12 +50867,25 @@
       <c r="BF6" s="3" t="n">
         <v>-1.396020413318183</v>
       </c>
-      <c r="BG6" s="2" t="inlineStr">
+      <c r="BG6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH6" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI6" s="2" t="n"/>
+      <c r="BJ6" s="2" t="n"/>
+      <c r="BK6" s="3" t="n">
+        <v>128.7270232293541</v>
+      </c>
+      <c r="BL6" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH6" s="2" t="b">
+      <c r="BM6" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -50337,12 +51036,10 @@
       <c r="AN7" s="2" t="n"/>
       <c r="AO7" s="2" t="inlineStr">
         <is>
-          <t>computed native-window/integrity bookkeeping; kinetic QC separate</t>
-        </is>
-      </c>
-      <c r="AP7" s="3" t="n">
-        <v>161.7060319318244</v>
-      </c>
+          <t>provisional model window/path estimate; phenothiazine_second_oxidation_unqualified</t>
+        </is>
+      </c>
+      <c r="AP7" s="2" t="n"/>
       <c r="AQ7" s="2" t="b">
         <v>0</v>
       </c>
@@ -50393,12 +51090,31 @@
       <c r="BF7" s="3" t="n">
         <v>1.460436998087971</v>
       </c>
-      <c r="BG7" s="2" t="inlineStr">
+      <c r="BG7" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH7" s="2" t="inlineStr">
+        <is>
+          <t>phenothiazine_second_oxidation_unqualified</t>
+        </is>
+      </c>
+      <c r="BI7" s="2" t="inlineStr">
+        <is>
+          <t>results/reviews/2026-10-19/phenothiazine_checked_subset/model_discrepancy.json</t>
+        </is>
+      </c>
+      <c r="BJ7" s="3" t="n">
+        <v>0.547</v>
+      </c>
+      <c r="BK7" s="3" t="n">
+        <v>161.7060319318244</v>
+      </c>
+      <c r="BL7" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH7" s="2" t="b">
+      <c r="BM7" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -50549,12 +51265,10 @@
       <c r="AN8" s="2" t="n"/>
       <c r="AO8" s="2" t="inlineStr">
         <is>
-          <t>computed native-window/integrity bookkeeping; kinetic QC separate</t>
-        </is>
-      </c>
-      <c r="AP8" s="3" t="n">
-        <v>157.9298261362036</v>
-      </c>
+          <t>provisional model window/path estimate; phenothiazine_second_oxidation_unqualified</t>
+        </is>
+      </c>
+      <c r="AP8" s="2" t="n"/>
       <c r="AQ8" s="2" t="b">
         <v>0</v>
       </c>
@@ -50605,12 +51319,31 @@
       <c r="BF8" s="3" t="n">
         <v>1.696166586334584</v>
       </c>
-      <c r="BG8" s="2" t="inlineStr">
+      <c r="BG8" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH8" s="2" t="inlineStr">
+        <is>
+          <t>phenothiazine_second_oxidation_unqualified</t>
+        </is>
+      </c>
+      <c r="BI8" s="2" t="inlineStr">
+        <is>
+          <t>results/reviews/2026-10-19/phenothiazine_checked_subset/model_discrepancy.json</t>
+        </is>
+      </c>
+      <c r="BJ8" s="3" t="n">
+        <v>0.547</v>
+      </c>
+      <c r="BK8" s="3" t="n">
+        <v>157.9298261362036</v>
+      </c>
+      <c r="BL8" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH8" s="2" t="b">
+      <c r="BM8" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -50833,12 +51566,25 @@
       <c r="BF9" s="3" t="n">
         <v>-1.218669026322459</v>
       </c>
-      <c r="BG9" s="2" t="inlineStr">
+      <c r="BG9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH9" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI9" s="2" t="n"/>
+      <c r="BJ9" s="2" t="n"/>
+      <c r="BK9" s="3" t="n">
+        <v>176.0724297272963</v>
+      </c>
+      <c r="BL9" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH9" s="2" t="b">
+      <c r="BM9" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -51061,12 +51807,25 @@
       <c r="BF10" s="3" t="n">
         <v>-1.097161965291889</v>
       </c>
-      <c r="BG10" s="2" t="inlineStr">
+      <c r="BG10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH10" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI10" s="2" t="n"/>
+      <c r="BJ10" s="2" t="n"/>
+      <c r="BK10" s="3" t="n">
+        <v>173.809864749964</v>
+      </c>
+      <c r="BL10" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH10" s="2" t="b">
+      <c r="BM10" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -51289,12 +52048,25 @@
       <c r="BF11" s="3" t="n">
         <v>-0.9784089635832061</v>
       </c>
-      <c r="BG11" s="2" t="inlineStr">
+      <c r="BG11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH11" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI11" s="2" t="n"/>
+      <c r="BJ11" s="2" t="n"/>
+      <c r="BK11" s="3" t="n">
+        <v>169.9415455230768</v>
+      </c>
+      <c r="BL11" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH11" s="2" t="b">
+      <c r="BM11" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -51517,12 +52289,25 @@
       <c r="BF12" s="3" t="n">
         <v>-1.229636791802477</v>
       </c>
-      <c r="BG12" s="2" t="inlineStr">
+      <c r="BG12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH12" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI12" s="2" t="n"/>
+      <c r="BJ12" s="2" t="n"/>
+      <c r="BK12" s="3" t="n">
+        <v>160.2657462526166</v>
+      </c>
+      <c r="BL12" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH12" s="2" t="b">
+      <c r="BM12" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -51745,12 +52530,25 @@
       <c r="BF13" s="3" t="n">
         <v>-1.961579773873382</v>
       </c>
-      <c r="BG13" s="2" t="inlineStr">
+      <c r="BG13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH13" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI13" s="2" t="n"/>
+      <c r="BJ13" s="2" t="n"/>
+      <c r="BK13" s="3" t="n">
+        <v>147.9171662427774</v>
+      </c>
+      <c r="BL13" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH13" s="2" t="b">
+      <c r="BM13" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -51973,12 +52771,25 @@
       <c r="BF14" s="3" t="n">
         <v>-1.812520659193979</v>
       </c>
-      <c r="BG14" s="2" t="inlineStr">
+      <c r="BG14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH14" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI14" s="2" t="n"/>
+      <c r="BJ14" s="2" t="n"/>
+      <c r="BK14" s="3" t="n">
+        <v>146.3170599781871</v>
+      </c>
+      <c r="BL14" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH14" s="2" t="b">
+      <c r="BM14" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -52201,12 +53012,25 @@
       <c r="BF15" s="3" t="n">
         <v>-1.766550722793909</v>
       </c>
-      <c r="BG15" s="2" t="inlineStr">
+      <c r="BG15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH15" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI15" s="2" t="n"/>
+      <c r="BJ15" s="2" t="n"/>
+      <c r="BK15" s="3" t="n">
+        <v>143.5660321422534</v>
+      </c>
+      <c r="BL15" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH15" s="2" t="b">
+      <c r="BM15" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -52429,12 +53253,25 @@
       <c r="BF16" s="3" t="n">
         <v>-2.044667244794255</v>
       </c>
-      <c r="BG16" s="2" t="inlineStr">
+      <c r="BG16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH16" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI16" s="2" t="n"/>
+      <c r="BJ16" s="2" t="n"/>
+      <c r="BK16" s="3" t="n">
+        <v>136.5990308347342</v>
+      </c>
+      <c r="BL16" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH16" s="2" t="b">
+      <c r="BM16" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -52657,12 +53494,25 @@
       <c r="BF17" s="3" t="n">
         <v>-1.413316320657032</v>
       </c>
-      <c r="BG17" s="2" t="inlineStr">
+      <c r="BG17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH17" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI17" s="2" t="n"/>
+      <c r="BJ17" s="2" t="n"/>
+      <c r="BK17" s="3" t="n">
+        <v>129.9639037662934</v>
+      </c>
+      <c r="BL17" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH17" s="2" t="b">
+      <c r="BM17" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -52885,12 +53735,25 @@
       <c r="BF18" s="3" t="n">
         <v>-1.382775743928505</v>
       </c>
-      <c r="BG18" s="2" t="inlineStr">
+      <c r="BG18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH18" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI18" s="2" t="n"/>
+      <c r="BJ18" s="2" t="n"/>
+      <c r="BK18" s="3" t="n">
+        <v>128.7270232293541</v>
+      </c>
+      <c r="BL18" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH18" s="2" t="b">
+      <c r="BM18" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -53113,12 +53976,25 @@
       <c r="BF19" s="3" t="n">
         <v>-1.180092339156545</v>
       </c>
-      <c r="BG19" s="2" t="inlineStr">
+      <c r="BG19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH19" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI19" s="2" t="n"/>
+      <c r="BJ19" s="2" t="n"/>
+      <c r="BK19" s="3" t="n">
+        <v>126.5928618062313</v>
+      </c>
+      <c r="BL19" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH19" s="2" t="b">
+      <c r="BM19" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -53341,12 +54217,25 @@
       <c r="BF20" s="3" t="n">
         <v>-1.47280520269851</v>
       </c>
-      <c r="BG20" s="2" t="inlineStr">
+      <c r="BG20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH20" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI20" s="2" t="n"/>
+      <c r="BJ20" s="2" t="n"/>
+      <c r="BK20" s="3" t="n">
+        <v>121.1445773596211</v>
+      </c>
+      <c r="BL20" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH20" s="2" t="b">
+      <c r="BM20" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -53569,12 +54458,25 @@
       <c r="BF21" s="3" t="n">
         <v>-1.255756395821663</v>
       </c>
-      <c r="BG21" s="2" t="inlineStr">
+      <c r="BG21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH21" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI21" s="2" t="n"/>
+      <c r="BJ21" s="2" t="n"/>
+      <c r="BK21" s="3" t="n">
+        <v>167.2813363320254</v>
+      </c>
+      <c r="BL21" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH21" s="2" t="b">
+      <c r="BM21" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -53797,12 +54699,25 @@
       <c r="BF22" s="3" t="n">
         <v>-1.240511492196674</v>
       </c>
-      <c r="BG22" s="2" t="inlineStr">
+      <c r="BG22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH22" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI22" s="2" t="n"/>
+      <c r="BJ22" s="2" t="n"/>
+      <c r="BK22" s="3" t="n">
+        <v>176.0724297272963</v>
+      </c>
+      <c r="BL22" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH22" s="2" t="b">
+      <c r="BM22" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -54025,12 +54940,25 @@
       <c r="BF23" s="3" t="n">
         <v>-1.924034197720175</v>
       </c>
-      <c r="BG23" s="2" t="inlineStr">
+      <c r="BG23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH23" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI23" s="2" t="n"/>
+      <c r="BJ23" s="2" t="n"/>
+      <c r="BK23" s="3" t="n">
+        <v>141.6628670580386</v>
+      </c>
+      <c r="BL23" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH23" s="2" t="b">
+      <c r="BM23" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -54253,12 +55181,25 @@
       <c r="BF24" s="3" t="n">
         <v>-1.959497902098519</v>
       </c>
-      <c r="BG24" s="2" t="inlineStr">
+      <c r="BG24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH24" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI24" s="2" t="n"/>
+      <c r="BJ24" s="2" t="n"/>
+      <c r="BK24" s="3" t="n">
+        <v>147.9171662427774</v>
+      </c>
+      <c r="BL24" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH24" s="2" t="b">
+      <c r="BM24" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -54481,12 +55422,25 @@
       <c r="BF25" s="3" t="n">
         <v>-1.507487979266443</v>
       </c>
-      <c r="BG25" s="2" t="inlineStr">
+      <c r="BG25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH25" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI25" s="2" t="n"/>
+      <c r="BJ25" s="2" t="n"/>
+      <c r="BK25" s="3" t="n">
+        <v>125.1107782788156</v>
+      </c>
+      <c r="BL25" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH25" s="2" t="b">
+      <c r="BM25" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -54709,17 +55663,30 @@
       <c r="BF26" s="3" t="n">
         <v>-1.473810802955995</v>
       </c>
-      <c r="BG26" s="2" t="inlineStr">
+      <c r="BG26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH26" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI26" s="2" t="n"/>
+      <c r="BJ26" s="2" t="n"/>
+      <c r="BK26" s="3" t="n">
+        <v>129.9639037662934</v>
+      </c>
+      <c r="BL26" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH26" s="2" t="b">
+      <c r="BM26" s="2" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BH26"/>
+  <autoFilter ref="A1:BM26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -54731,7 +55698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH2"/>
+  <dimension ref="A1:BM2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -54793,7 +55760,12 @@
     <col width="22" customWidth="1" min="57" max="57"/>
     <col width="22" customWidth="1" min="58" max="58"/>
     <col width="22" customWidth="1" min="59" max="59"/>
-    <col width="22" customWidth="1" min="60" max="60"/>
+    <col width="35" customWidth="1" min="60" max="60"/>
+    <col width="22" customWidth="1" min="61" max="61"/>
+    <col width="22" customWidth="1" min="62" max="62"/>
+    <col width="22" customWidth="1" min="63" max="63"/>
+    <col width="22" customWidth="1" min="64" max="64"/>
+    <col width="22" customWidth="1" min="65" max="65"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -55089,10 +56061,35 @@
       </c>
       <c r="BG1" s="1" t="inlineStr">
         <is>
+          <t>model_primary_admissible</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>model_validation_status</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>model_validation_evidence</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>model_max_observed_error_V</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>model_accessible_capacity_estimate_mAh_g</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
           <t>fleet_progress</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
         <is>
           <t>experimentally_validated_for_exact_graft</t>
         </is>
@@ -55289,17 +56286,30 @@
       <c r="BF2" s="3" t="n">
         <v>-1.198326265264768</v>
       </c>
-      <c r="BG2" s="2" t="inlineStr">
+      <c r="BG2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH2" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI2" s="2" t="n"/>
+      <c r="BJ2" s="2" t="n"/>
+      <c r="BK2" s="3" t="n">
+        <v>184.5768475220856</v>
+      </c>
+      <c r="BL2" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
         </is>
       </c>
-      <c r="BH2" s="2" t="b">
+      <c r="BM2" s="2" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BH2"/>
+  <autoFilter ref="A1:BM2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -56273,7 +57283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -56288,7 +57298,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-19T05:49:46.921559-05:00</t>
+          <t>2026-10-19T06:24:53.538237-05:00</t>
         </is>
       </c>
     </row>
@@ -56324,125 +57334,149 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Native potential window and integrity-contiguous path bookkeeping; kinetics assessed separately.</t>
+          <t>Native potential window and integrity-contiguous path bookkeeping, withheld where a scoped model limitation applies; kinetics assessed separately.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>gas_Nelsen_sum_eV</t>
+          <t>model_accessible_capacity_estimate_mAh_g</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Only QC-clean current-protocol four-point GAS diagnostic; never a validated solution rate or full solution reorganization energy.</t>
+          <t>Original model window/path estimate retained for diagnosis; not qualified capacity when model_primary_admissible is false.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>empty_numeric_cells</t>
+          <t>model_max_observed_error_V</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pending, flagged or not independently admissible. Never substituted parent/zero values.</t>
+          <t>Largest reviewed free-parent residual for the scoped model limitation; never a measurement or error bound for an exact graft.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>experimental_accuracy</t>
+          <t>gas_Nelsen_sum_eV</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>No exact graft has an experimentally validated property in this dataset.</t>
+          <t>Only QC-clean current-protocol four-point GAS diagnostic; never a validated solution rate or full solution reorganization energy.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>paired_shifts</t>
+          <t>empty_numeric_cells</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Candidate minus declared exact-graft control, same charge/electron ladder and snapshot. Each event requires two admitted values; no surface/parent substitution or improvement claim.</t>
+          <t>Pending, flagged or not independently admissible. Never substituted parent/zero values.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>spin_qc</t>
+          <t>experimental_accuracy</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UMA gaps&lt;0.5eV require DFT alternatives; DFT electronic gaps within0.2eV require matching native spin thermals; native gaps within0.1eV require spin-ensemble evaluation. Raw surfaces remain diagnostics; far positive electronic gaps retain explicit thermal uncertainty.</t>
+          <t>No exact graft has an experimentally validated property in this dataset.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>native_g_thermal_eV</t>
+          <t>paired_shifts</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Corrected native partition of the selected single spin surface, before any equilibrium mixing correction.</t>
+          <t>Candidate minus declared exact-graft control, same charge/electron ladder and snapshot. Each event requires two admitted values; no surface/parent substitution or improvement claim.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>effective_g_thermal_eV</t>
+          <t>spin_qc</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Native term added to the selected active SMD energy; includes an admitted equilibrium spin correction when selected.</t>
+          <t>UMA gaps&lt;0.5eV require DFT alternatives; DFT electronic gaps within0.2eV require matching native spin thermals; native gaps within0.1eV require spin-ensemble evaluation. Raw surfaces remain diagnostics; far positive electronic gaps retain explicit thermal uncertainty.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>spin_ensemble_correction_eV</t>
+          <t>native_g_thermal_eV</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Equilibrium G minus selected-surface G. Component spin degeneracy is included once, not multiplied again.</t>
+          <t>Corrected native partition of the selected single spin surface, before any equilibrium mixing correction.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>spin_ensemble_alternative_population</t>
+          <t>effective_g_thermal_eV</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Alternative-spin equilibrium population at 298.15 K under the selected two-spin model; this does not validate kinetics.</t>
+          <t>Native term added to the selected active SMD energy; includes an admitted equilibrium spin correction when selected.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>spin_ensemble_correction_eV</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Equilibrium G minus selected-surface G. Component spin degeneracy is included once, not multiplied again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>spin_ensemble_alternative_population</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Alternative-spin equilibrium population at 298.15 K under the selected two-spin model; this does not validate kinetics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>workbook</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Immutable snapshot of independently audited external pipeline records, no spreadsheet formulas.</t>
         </is>

</xml_diff>

<commit_message>
Register cata-imide designs and start six reserved solution-state calculations
</commit_message>
<xml_diff>
--- a/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
+++ b/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
@@ -17,11 +17,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Original39'!$A$1:$BM$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'States'!$A$1:$AL$194</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Couples'!$A$1:$T$129</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Additional'!$A$1:$BM$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'States'!$A$1:$AL$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Couples'!$A$1:$T$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Additional'!$A$1:$BM$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Controls'!$A$1:$BM$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Comparisons'!$A$1:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Comparisons'!$A$1:$I$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -11085,7 +11085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL194"/>
+  <dimension ref="A1:AL200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -38533,26 +38533,26 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>ethylviologen</t>
+          <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>MYJMGLDZQAZLCC-UHFFFAOYSA-N</t>
+          <t>NANYKQXYZMYUQE-UHFFFAOYSA-N</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>ethylviologen</t>
+          <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>ox2</t>
+          <t>neu</t>
         </is>
       </c>
       <c r="E192" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F192" s="2" t="n">
         <v>1</v>
@@ -38568,14 +38568,16 @@
           <t>verified graph/warm start</t>
         </is>
       </c>
-      <c r="J192" s="2" t="n"/>
-      <c r="K192" s="4" t="inlineStr">
-        <is>
-          <t>legacy; rerun required</t>
+      <c r="J192" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K192" s="2" t="inlineStr">
+        <is>
+          <t>fingerprinted</t>
         </is>
       </c>
       <c r="L192" s="3" t="n">
-        <v>-24063.02741162595</v>
+        <v>-36353.14200248472</v>
       </c>
       <c r="M192" s="2" t="n">
         <v>1</v>
@@ -38586,64 +38588,48 @@
         </is>
       </c>
       <c r="O192" s="3" t="n">
-        <v>0.01834559999406338</v>
+        <v>0.01897270977497101</v>
       </c>
       <c r="P192" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q192" s="2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="R192" s="3" t="n">
-        <v>-24070.13276285656</v>
-      </c>
-      <c r="S192" s="2" t="inlineStr">
-        <is>
-          <t>addressed QC passed</t>
-        </is>
-      </c>
-      <c r="T192" s="3" t="n">
-        <v>8.967428730909329</v>
-      </c>
-      <c r="U192" s="3" t="n">
-        <v>8.967428730909329</v>
-      </c>
-      <c r="V192" s="2" t="inlineStr">
-        <is>
-          <t>not_selected</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q192" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="R192" s="2" t="n"/>
+      <c r="S192" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="T192" s="2" t="n"/>
+      <c r="U192" s="2" t="n"/>
+      <c r="V192" s="2" t="n"/>
       <c r="W192" s="2" t="n"/>
       <c r="X192" s="2" t="n"/>
-      <c r="Y192" s="2" t="inlineStr">
-        <is>
-          <t>native_solution_dft_qrrho_spin</t>
-        </is>
-      </c>
+      <c r="Y192" s="2" t="n"/>
       <c r="Z192" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
-        </is>
-      </c>
-      <c r="AA192" s="2" t="inlineStr"/>
-      <c r="AB192" s="3" t="n">
-        <v>-24061.16533412565</v>
-      </c>
-      <c r="AC192" s="2" t="inlineStr">
-        <is>
-          <t>verified calculation</t>
-        </is>
-      </c>
-      <c r="AD192" s="2" t="inlineStr">
-        <is>
-          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/ethylviologen/ox2/result.json</t>
-        </is>
-      </c>
+          <t>INCOMPLETE</t>
+        </is>
+      </c>
+      <c r="AA192" s="2" t="inlineStr">
+        <is>
+          <t>missing_geometry_or_result</t>
+        </is>
+      </c>
+      <c r="AB192" s="2" t="n"/>
+      <c r="AC192" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AD192" s="2" t="n"/>
       <c r="AE192" s="2" t="inlineStr">
         <is>
-          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/ox2/result.json</t>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_ndi_ethyl/neu/result.json</t>
         </is>
       </c>
       <c r="AF192" s="2" t="inlineStr">
@@ -38652,7 +38638,7 @@
         </is>
       </c>
       <c r="AG192" s="3" t="n">
-        <v>2.3433</v>
+        <v>2.361</v>
       </c>
       <c r="AH192" s="2" t="inlineStr">
         <is>
@@ -38661,40 +38647,38 @@
       </c>
       <c r="AI192" s="2" t="inlineStr">
         <is>
-          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/ox2/result.json</t>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_ndi_ethyl/neu/result.json</t>
         </is>
       </c>
       <c r="AJ192" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK192" s="3" t="n">
-        <v>-24061.16533412565</v>
-      </c>
+      <c r="AK192" s="2" t="n"/>
       <c r="AL192" s="2" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>ethylviologen</t>
+          <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>MYJMGLDZQAZLCC-UHFFFAOYSA-N</t>
+          <t>NANYKQXYZMYUQE-UHFFFAOYSA-N</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>ethylviologen</t>
+          <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>ox1</t>
+          <t>red1</t>
         </is>
       </c>
       <c r="E193" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F193" s="2" t="n">
         <v>2</v>
@@ -38710,14 +38694,16 @@
           <t>verified graph/warm start</t>
         </is>
       </c>
-      <c r="J193" s="2" t="n"/>
-      <c r="K193" s="4" t="inlineStr">
-        <is>
-          <t>legacy; rerun required</t>
+      <c r="J193" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K193" s="2" t="inlineStr">
+        <is>
+          <t>fingerprinted</t>
         </is>
       </c>
       <c r="L193" s="3" t="n">
-        <v>-24071.5215716843</v>
+        <v>-36355.05412454171</v>
       </c>
       <c r="M193" s="2" t="n">
         <v>2</v>
@@ -38728,64 +38714,48 @@
         </is>
       </c>
       <c r="O193" s="3" t="n">
-        <v>0.01841003447771072</v>
+        <v>0.01764801330864429</v>
       </c>
       <c r="P193" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q193" s="2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="R193" s="3" t="n">
-        <v>-24073.79072358517</v>
-      </c>
-      <c r="S193" s="2" t="inlineStr">
-        <is>
-          <t>addressed QC passed</t>
-        </is>
-      </c>
-      <c r="T193" s="3" t="n">
-        <v>8.867693688416539</v>
-      </c>
-      <c r="U193" s="3" t="n">
-        <v>8.867693688416539</v>
-      </c>
-      <c r="V193" s="2" t="inlineStr">
-        <is>
-          <t>not_selected</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q193" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="R193" s="2" t="n"/>
+      <c r="S193" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="T193" s="2" t="n"/>
+      <c r="U193" s="2" t="n"/>
+      <c r="V193" s="2" t="n"/>
       <c r="W193" s="2" t="n"/>
       <c r="X193" s="2" t="n"/>
-      <c r="Y193" s="2" t="inlineStr">
-        <is>
-          <t>native_solution_dft_qrrho_spin</t>
-        </is>
-      </c>
+      <c r="Y193" s="2" t="n"/>
       <c r="Z193" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
-        </is>
-      </c>
-      <c r="AA193" s="2" t="inlineStr"/>
-      <c r="AB193" s="3" t="n">
-        <v>-24064.92302989676</v>
-      </c>
-      <c r="AC193" s="2" t="inlineStr">
-        <is>
-          <t>verified calculation</t>
-        </is>
-      </c>
-      <c r="AD193" s="2" t="inlineStr">
-        <is>
-          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/ethylviologen/ox1/result.json</t>
-        </is>
-      </c>
+          <t>INCOMPLETE</t>
+        </is>
+      </c>
+      <c r="AA193" s="2" t="inlineStr">
+        <is>
+          <t>missing_geometry_or_result</t>
+        </is>
+      </c>
+      <c r="AB193" s="2" t="n"/>
+      <c r="AC193" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AD193" s="2" t="n"/>
       <c r="AE193" s="2" t="inlineStr">
         <is>
-          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/ox1/result.json</t>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_ndi_ethyl/red1/result.json</t>
         </is>
       </c>
       <c r="AF193" s="2" t="inlineStr">
@@ -38801,40 +38771,38 @@
       </c>
       <c r="AI193" s="2" t="inlineStr">
         <is>
-          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/ox1/result.json</t>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_ndi_ethyl/red1/result.json</t>
         </is>
       </c>
       <c r="AJ193" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK193" s="3" t="n">
-        <v>-24064.92302989676</v>
-      </c>
+      <c r="AK193" s="2" t="n"/>
       <c r="AL193" s="2" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>ethylviologen</t>
+          <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>MYJMGLDZQAZLCC-UHFFFAOYSA-N</t>
+          <t>NANYKQXYZMYUQE-UHFFFAOYSA-N</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>ethylviologen</t>
+          <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>neu</t>
+          <t>red2</t>
         </is>
       </c>
       <c r="E194" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="F194" s="2" t="n">
         <v>1</v>
@@ -38850,14 +38818,16 @@
           <t>verified graph/warm start</t>
         </is>
       </c>
-      <c r="J194" s="2" t="n"/>
-      <c r="K194" s="4" t="inlineStr">
-        <is>
-          <t>legacy; rerun required</t>
+      <c r="J194" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K194" s="2" t="inlineStr">
+        <is>
+          <t>fingerprinted</t>
         </is>
       </c>
       <c r="L194" s="3" t="n">
-        <v>-24076.15347061308</v>
+        <v>-36353.30121007407</v>
       </c>
       <c r="M194" s="2" t="n">
         <v>1</v>
@@ -38868,73 +38838,57 @@
         </is>
       </c>
       <c r="O194" s="3" t="n">
-        <v>0.01812604255974293</v>
+        <v>0.01944873854517937</v>
       </c>
       <c r="P194" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q194" s="2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="R194" s="3" t="n">
-        <v>-24076.88021424419</v>
-      </c>
-      <c r="S194" s="2" t="inlineStr">
-        <is>
-          <t>addressed QC passed</t>
-        </is>
-      </c>
-      <c r="T194" s="3" t="n">
-        <v>8.776314711099106</v>
-      </c>
-      <c r="U194" s="3" t="n">
-        <v>8.776314711099106</v>
-      </c>
-      <c r="V194" s="2" t="inlineStr">
-        <is>
-          <t>not_selected</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q194" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="R194" s="2" t="n"/>
+      <c r="S194" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="T194" s="2" t="n"/>
+      <c r="U194" s="2" t="n"/>
+      <c r="V194" s="2" t="n"/>
       <c r="W194" s="2" t="n"/>
       <c r="X194" s="2" t="n"/>
-      <c r="Y194" s="2" t="inlineStr">
-        <is>
-          <t>native_solution_dft_qrrho_spin</t>
-        </is>
-      </c>
+      <c r="Y194" s="2" t="n"/>
       <c r="Z194" s="2" t="inlineStr">
         <is>
-          <t>ready</t>
-        </is>
-      </c>
-      <c r="AA194" s="2" t="inlineStr"/>
-      <c r="AB194" s="3" t="n">
-        <v>-24068.10389953309</v>
-      </c>
-      <c r="AC194" s="2" t="inlineStr">
-        <is>
-          <t>verified calculation</t>
-        </is>
-      </c>
-      <c r="AD194" s="2" t="inlineStr">
-        <is>
-          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/ethylviologen/neu/result.json</t>
-        </is>
-      </c>
+          <t>INCOMPLETE</t>
+        </is>
+      </c>
+      <c r="AA194" s="2" t="inlineStr">
+        <is>
+          <t>missing_geometry_or_result</t>
+        </is>
+      </c>
+      <c r="AB194" s="2" t="n"/>
+      <c r="AC194" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AD194" s="2" t="n"/>
       <c r="AE194" s="2" t="inlineStr">
         <is>
-          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/neu/result.json</t>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_ndi_ethyl/red2/result.json</t>
         </is>
       </c>
       <c r="AF194" s="2" t="inlineStr">
         <is>
-          <t>UMA_large_gap_preliminary</t>
+          <t>DFT_check_required</t>
         </is>
       </c>
       <c r="AG194" s="3" t="n">
-        <v>1.3246</v>
+        <v>0.2348</v>
       </c>
       <c r="AH194" s="2" t="inlineStr">
         <is>
@@ -38943,19 +38897,817 @@
       </c>
       <c r="AI194" s="2" t="inlineStr">
         <is>
-          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/neu/result.json</t>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_ndi_ethyl/red2/result.json</t>
         </is>
       </c>
       <c r="AJ194" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK194" s="3" t="n">
-        <v>-24068.10389953309</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AK194" s="2" t="n"/>
       <c r="AL194" s="2" t="n"/>
     </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>LKTOOBTUSSFQCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="E195" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F195" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G195" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H195" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I195" s="2" t="inlineStr">
+        <is>
+          <t>verified graph/warm start</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
+          <t>fingerprinted</t>
+        </is>
+      </c>
+      <c r="L195" s="3" t="n">
+        <v>-40533.80453061792</v>
+      </c>
+      <c r="M195" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N195" s="2" t="inlineStr">
+        <is>
+          <t>uma-s-1p2p1</t>
+        </is>
+      </c>
+      <c r="O195" s="3" t="n">
+        <v>0.01762303523719311</v>
+      </c>
+      <c r="P195" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q195" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="R195" s="2" t="n"/>
+      <c r="S195" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="T195" s="2" t="n"/>
+      <c r="U195" s="2" t="n"/>
+      <c r="V195" s="2" t="n"/>
+      <c r="W195" s="2" t="n"/>
+      <c r="X195" s="2" t="n"/>
+      <c r="Y195" s="2" t="n"/>
+      <c r="Z195" s="2" t="inlineStr">
+        <is>
+          <t>INCOMPLETE</t>
+        </is>
+      </c>
+      <c r="AA195" s="2" t="inlineStr">
+        <is>
+          <t>missing_geometry_or_result</t>
+        </is>
+      </c>
+      <c r="AB195" s="2" t="n"/>
+      <c r="AC195" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AD195" s="2" t="n"/>
+      <c r="AE195" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_adi_ethyl/neu/result.json</t>
+        </is>
+      </c>
+      <c r="AF195" s="2" t="inlineStr">
+        <is>
+          <t>UMA_large_gap_preliminary</t>
+        </is>
+      </c>
+      <c r="AG195" s="3" t="n">
+        <v>1.6917</v>
+      </c>
+      <c r="AH195" s="2" t="inlineStr">
+        <is>
+          <t>UMA gas preoptimization; solution ground state not independently established</t>
+        </is>
+      </c>
+      <c r="AI195" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_adi_ethyl/neu/result.json</t>
+        </is>
+      </c>
+      <c r="AJ195" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK195" s="2" t="n"/>
+      <c r="AL195" s="2" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>LKTOOBTUSSFQCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>red1</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F196" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G196" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H196" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>verified graph/warm start</t>
+        </is>
+      </c>
+      <c r="J196" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K196" s="2" t="inlineStr">
+        <is>
+          <t>fingerprinted</t>
+        </is>
+      </c>
+      <c r="L196" s="3" t="n">
+        <v>-40535.94089269378</v>
+      </c>
+      <c r="M196" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N196" s="2" t="inlineStr">
+        <is>
+          <t>uma-s-1p2p1</t>
+        </is>
+      </c>
+      <c r="O196" s="3" t="n">
+        <v>0.014229373075068</v>
+      </c>
+      <c r="P196" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q196" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="R196" s="2" t="n"/>
+      <c r="S196" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="T196" s="2" t="n"/>
+      <c r="U196" s="2" t="n"/>
+      <c r="V196" s="2" t="n"/>
+      <c r="W196" s="2" t="n"/>
+      <c r="X196" s="2" t="n"/>
+      <c r="Y196" s="2" t="n"/>
+      <c r="Z196" s="2" t="inlineStr">
+        <is>
+          <t>INCOMPLETE</t>
+        </is>
+      </c>
+      <c r="AA196" s="2" t="inlineStr">
+        <is>
+          <t>missing_geometry_or_result</t>
+        </is>
+      </c>
+      <c r="AB196" s="2" t="n"/>
+      <c r="AC196" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AD196" s="2" t="n"/>
+      <c r="AE196" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_adi_ethyl/red1/result.json</t>
+        </is>
+      </c>
+      <c r="AF196" s="2" t="inlineStr">
+        <is>
+          <t>standard_doublet_model</t>
+        </is>
+      </c>
+      <c r="AG196" s="2" t="n"/>
+      <c r="AH196" s="2" t="inlineStr">
+        <is>
+          <t>electron parity / no alternative scan</t>
+        </is>
+      </c>
+      <c r="AI196" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_adi_ethyl/red1/result.json</t>
+        </is>
+      </c>
+      <c r="AJ196" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK196" s="2" t="n"/>
+      <c r="AL196" s="2" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>LKTOOBTUSSFQCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>red2</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F197" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G197" s="2" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H197" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I197" s="2" t="inlineStr">
+        <is>
+          <t>verified graph/warm start</t>
+        </is>
+      </c>
+      <c r="J197" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K197" s="2" t="inlineStr">
+        <is>
+          <t>fingerprinted</t>
+        </is>
+      </c>
+      <c r="L197" s="3" t="n">
+        <v>-40534.59472504167</v>
+      </c>
+      <c r="M197" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N197" s="2" t="inlineStr">
+        <is>
+          <t>uma-s-1p2p1</t>
+        </is>
+      </c>
+      <c r="O197" s="3" t="n">
+        <v>0.01947363466024399</v>
+      </c>
+      <c r="P197" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q197" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="R197" s="2" t="n"/>
+      <c r="S197" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="T197" s="2" t="n"/>
+      <c r="U197" s="2" t="n"/>
+      <c r="V197" s="2" t="n"/>
+      <c r="W197" s="2" t="n"/>
+      <c r="X197" s="2" t="n"/>
+      <c r="Y197" s="2" t="n"/>
+      <c r="Z197" s="2" t="inlineStr">
+        <is>
+          <t>INCOMPLETE</t>
+        </is>
+      </c>
+      <c r="AA197" s="2" t="inlineStr">
+        <is>
+          <t>missing_geometry_or_result</t>
+        </is>
+      </c>
+      <c r="AB197" s="2" t="n"/>
+      <c r="AC197" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AD197" s="2" t="n"/>
+      <c r="AE197" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_adi_ethyl/red2/result.json</t>
+        </is>
+      </c>
+      <c r="AF197" s="2" t="inlineStr">
+        <is>
+          <t>UMA_large_gap_preliminary</t>
+        </is>
+      </c>
+      <c r="AG197" s="3" t="n">
+        <v>0.5248</v>
+      </c>
+      <c r="AH197" s="2" t="inlineStr">
+        <is>
+          <t>UMA gas preoptimization; solution ground state not independently established</t>
+        </is>
+      </c>
+      <c r="AI197" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_adi_ethyl/red2/result.json</t>
+        </is>
+      </c>
+      <c r="AJ197" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK197" s="2" t="n"/>
+      <c r="AL197" s="2" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>ethylviologen</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>MYJMGLDZQAZLCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>ethylviologen</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>ox2</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F198" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G198" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H198" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I198" s="2" t="inlineStr">
+        <is>
+          <t>verified graph/warm start</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="n"/>
+      <c r="K198" s="4" t="inlineStr">
+        <is>
+          <t>legacy; rerun required</t>
+        </is>
+      </c>
+      <c r="L198" s="3" t="n">
+        <v>-24063.02741162595</v>
+      </c>
+      <c r="M198" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N198" s="2" t="inlineStr">
+        <is>
+          <t>uma-s-1p2p1</t>
+        </is>
+      </c>
+      <c r="O198" s="3" t="n">
+        <v>0.01834559999406338</v>
+      </c>
+      <c r="P198" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q198" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R198" s="3" t="n">
+        <v>-24070.13276285656</v>
+      </c>
+      <c r="S198" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T198" s="3" t="n">
+        <v>8.967428730909329</v>
+      </c>
+      <c r="U198" s="3" t="n">
+        <v>8.967428730909329</v>
+      </c>
+      <c r="V198" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="W198" s="2" t="n"/>
+      <c r="X198" s="2" t="n"/>
+      <c r="Y198" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
+      <c r="Z198" s="2" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA198" s="2" t="inlineStr"/>
+      <c r="AB198" s="3" t="n">
+        <v>-24061.16533412565</v>
+      </c>
+      <c r="AC198" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD198" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/ethylviologen/ox2/result.json</t>
+        </is>
+      </c>
+      <c r="AE198" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/ox2/result.json</t>
+        </is>
+      </c>
+      <c r="AF198" s="2" t="inlineStr">
+        <is>
+          <t>UMA_large_gap_preliminary</t>
+        </is>
+      </c>
+      <c r="AG198" s="3" t="n">
+        <v>2.3433</v>
+      </c>
+      <c r="AH198" s="2" t="inlineStr">
+        <is>
+          <t>UMA gas preoptimization; solution ground state not independently established</t>
+        </is>
+      </c>
+      <c r="AI198" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/ox2/result.json</t>
+        </is>
+      </c>
+      <c r="AJ198" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK198" s="3" t="n">
+        <v>-24061.16533412565</v>
+      </c>
+      <c r="AL198" s="2" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>ethylviologen</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>MYJMGLDZQAZLCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>ethylviologen</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>ox1</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F199" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G199" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H199" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I199" s="2" t="inlineStr">
+        <is>
+          <t>verified graph/warm start</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="n"/>
+      <c r="K199" s="4" t="inlineStr">
+        <is>
+          <t>legacy; rerun required</t>
+        </is>
+      </c>
+      <c r="L199" s="3" t="n">
+        <v>-24071.5215716843</v>
+      </c>
+      <c r="M199" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N199" s="2" t="inlineStr">
+        <is>
+          <t>uma-s-1p2p1</t>
+        </is>
+      </c>
+      <c r="O199" s="3" t="n">
+        <v>0.01841003447771072</v>
+      </c>
+      <c r="P199" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q199" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R199" s="3" t="n">
+        <v>-24073.79072358517</v>
+      </c>
+      <c r="S199" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T199" s="3" t="n">
+        <v>8.867693688416539</v>
+      </c>
+      <c r="U199" s="3" t="n">
+        <v>8.867693688416539</v>
+      </c>
+      <c r="V199" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="W199" s="2" t="n"/>
+      <c r="X199" s="2" t="n"/>
+      <c r="Y199" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
+      <c r="Z199" s="2" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA199" s="2" t="inlineStr"/>
+      <c r="AB199" s="3" t="n">
+        <v>-24064.92302989676</v>
+      </c>
+      <c r="AC199" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD199" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/ethylviologen/ox1/result.json</t>
+        </is>
+      </c>
+      <c r="AE199" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/ox1/result.json</t>
+        </is>
+      </c>
+      <c r="AF199" s="2" t="inlineStr">
+        <is>
+          <t>standard_doublet_model</t>
+        </is>
+      </c>
+      <c r="AG199" s="2" t="n"/>
+      <c r="AH199" s="2" t="inlineStr">
+        <is>
+          <t>electron parity / no alternative scan</t>
+        </is>
+      </c>
+      <c r="AI199" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/ox1/result.json</t>
+        </is>
+      </c>
+      <c r="AJ199" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK199" s="3" t="n">
+        <v>-24064.92302989676</v>
+      </c>
+      <c r="AL199" s="2" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>ethylviologen</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>MYJMGLDZQAZLCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>ethylviologen</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F200" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G200" s="2" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H200" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t>verified graph/warm start</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="n"/>
+      <c r="K200" s="4" t="inlineStr">
+        <is>
+          <t>legacy; rerun required</t>
+        </is>
+      </c>
+      <c r="L200" s="3" t="n">
+        <v>-24076.15347061308</v>
+      </c>
+      <c r="M200" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N200" s="2" t="inlineStr">
+        <is>
+          <t>uma-s-1p2p1</t>
+        </is>
+      </c>
+      <c r="O200" s="3" t="n">
+        <v>0.01812604255974293</v>
+      </c>
+      <c r="P200" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q200" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R200" s="3" t="n">
+        <v>-24076.88021424419</v>
+      </c>
+      <c r="S200" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T200" s="3" t="n">
+        <v>8.776314711099106</v>
+      </c>
+      <c r="U200" s="3" t="n">
+        <v>8.776314711099106</v>
+      </c>
+      <c r="V200" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="W200" s="2" t="n"/>
+      <c r="X200" s="2" t="n"/>
+      <c r="Y200" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
+      <c r="Z200" s="2" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA200" s="2" t="inlineStr"/>
+      <c r="AB200" s="3" t="n">
+        <v>-24068.10389953309</v>
+      </c>
+      <c r="AC200" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD200" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/ethylviologen/neu/result.json</t>
+        </is>
+      </c>
+      <c r="AE200" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/neu/result.json</t>
+        </is>
+      </c>
+      <c r="AF200" s="2" t="inlineStr">
+        <is>
+          <t>UMA_large_gap_preliminary</t>
+        </is>
+      </c>
+      <c r="AG200" s="3" t="n">
+        <v>1.3246</v>
+      </c>
+      <c r="AH200" s="2" t="inlineStr">
+        <is>
+          <t>UMA gas preoptimization; solution ground state not independently established</t>
+        </is>
+      </c>
+      <c r="AI200" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/ethylviologen/neu/result.json</t>
+        </is>
+      </c>
+      <c r="AJ200" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK200" s="3" t="n">
+        <v>-24068.10389953309</v>
+      </c>
+      <c r="AL200" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AL194"/>
+  <autoFilter ref="A1:AL200"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -38967,7 +39719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T129"/>
+  <dimension ref="A1:T133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -49217,51 +49969,43 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>ethylviologen</t>
+          <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>ethylviologen</t>
+          <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>MYJMGLDZQAZLCC-UHFFFAOYSA-N</t>
+          <t>NANYKQXYZMYUQE-UHFFFAOYSA-N</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>ox2-&gt;ox1</t>
+          <t>neu-&gt;red1</t>
         </is>
       </c>
       <c r="E128" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F128" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G128" s="3" t="n">
-        <v>-0.6215001304808538</v>
-      </c>
-      <c r="H128" s="2" t="inlineStr">
-        <is>
-          <t>native calculated/QC passed</t>
-        </is>
-      </c>
-      <c r="I128" s="2" t="inlineStr">
-        <is>
-          <t>intact_bound</t>
-        </is>
-      </c>
-      <c r="J128" s="3" t="n">
-        <v>3.658</v>
-      </c>
-      <c r="K128" s="2" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="G128" s="2" t="n"/>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I128" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="n"/>
+      <c r="K128" s="2" t="n"/>
       <c r="L128" s="2" t="n"/>
       <c r="M128" s="2" t="n"/>
       <c r="N128" s="2" t="n"/>
@@ -49288,58 +50032,48 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="T128" s="3" t="n">
-        <v>-0.6215001304808538</v>
-      </c>
+      <c r="T128" s="2" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>ethylviologen</t>
+          <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>ethylviologen</t>
+          <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>MYJMGLDZQAZLCC-UHFFFAOYSA-N</t>
+          <t>NANYKQXYZMYUQE-UHFFFAOYSA-N</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>ox1-&gt;neu</t>
+          <t>red1-&gt;red2</t>
         </is>
       </c>
       <c r="E129" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F129" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G129" s="3" t="n">
-        <v>-1.198326265264768</v>
-      </c>
+        <v>-2</v>
+      </c>
+      <c r="G129" s="2" t="n"/>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>native calculated/QC passed</t>
-        </is>
-      </c>
-      <c r="I129" s="2" t="inlineStr">
-        <is>
-          <t>intact_bound</t>
-        </is>
-      </c>
-      <c r="J129" s="3" t="n">
-        <v>3.089</v>
-      </c>
-      <c r="K129" s="2" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
+          <t>pending DFT spin validation</t>
+        </is>
+      </c>
+      <c r="I129" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="n"/>
+      <c r="K129" s="2" t="n"/>
       <c r="L129" s="2" t="n"/>
       <c r="M129" s="2" t="n"/>
       <c r="N129" s="2" t="n"/>
@@ -49363,15 +50097,305 @@
       </c>
       <c r="S129" s="2" t="inlineStr">
         <is>
+          <t>DFT spin validation required/wrong ground state</t>
+        </is>
+      </c>
+      <c r="T129" s="2" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>LKTOOBTUSSFQCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>neu-&gt;red1</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G130" s="2" t="n"/>
+      <c r="H130" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I130" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="n"/>
+      <c r="K130" s="2" t="n"/>
+      <c r="L130" s="2" t="n"/>
+      <c r="M130" s="2" t="n"/>
+      <c r="N130" s="2" t="n"/>
+      <c r="O130" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="P130" s="2" t="inlineStr">
+        <is>
+          <t>pending separate validated solution method</t>
+        </is>
+      </c>
+      <c r="Q130" s="2" t="inlineStr">
+        <is>
+          <t>pending separate validated solution method</t>
+        </is>
+      </c>
+      <c r="R130" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S130" s="2" t="inlineStr">
+        <is>
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="T129" s="3" t="n">
+      <c r="T130" s="2" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>LKTOOBTUSSFQCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>red1-&gt;red2</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F131" s="2" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G131" s="2" t="n"/>
+      <c r="H131" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I131" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="n"/>
+      <c r="K131" s="2" t="n"/>
+      <c r="L131" s="2" t="n"/>
+      <c r="M131" s="2" t="n"/>
+      <c r="N131" s="2" t="n"/>
+      <c r="O131" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="P131" s="2" t="inlineStr">
+        <is>
+          <t>pending separate validated solution method</t>
+        </is>
+      </c>
+      <c r="Q131" s="2" t="inlineStr">
+        <is>
+          <t>pending separate validated solution method</t>
+        </is>
+      </c>
+      <c r="R131" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S131" s="2" t="inlineStr">
+        <is>
+          <t>admissible under stated spin evidence</t>
+        </is>
+      </c>
+      <c r="T131" s="2" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>ethylviologen</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>ethylviologen</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>MYJMGLDZQAZLCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>ox2-&gt;ox1</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F132" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G132" s="3" t="n">
+        <v>-0.6215001304808538</v>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J132" s="3" t="n">
+        <v>3.658</v>
+      </c>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="L132" s="2" t="n"/>
+      <c r="M132" s="2" t="n"/>
+      <c r="N132" s="2" t="n"/>
+      <c r="O132" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="P132" s="2" t="inlineStr">
+        <is>
+          <t>pending separate validated solution method</t>
+        </is>
+      </c>
+      <c r="Q132" s="2" t="inlineStr">
+        <is>
+          <t>pending separate validated solution method</t>
+        </is>
+      </c>
+      <c r="R132" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S132" s="2" t="inlineStr">
+        <is>
+          <t>admissible under stated spin evidence</t>
+        </is>
+      </c>
+      <c r="T132" s="3" t="n">
+        <v>-0.6215001304808538</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>ethylviologen</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>ethylviologen</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>MYJMGLDZQAZLCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>ox1-&gt;neu</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F133" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G133" s="3" t="n">
+        <v>-1.198326265264768</v>
+      </c>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J133" s="3" t="n">
+        <v>3.089</v>
+      </c>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="L133" s="2" t="n"/>
+      <c r="M133" s="2" t="n"/>
+      <c r="N133" s="2" t="n"/>
+      <c r="O133" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="P133" s="2" t="inlineStr">
+        <is>
+          <t>pending separate validated solution method</t>
+        </is>
+      </c>
+      <c r="Q133" s="2" t="inlineStr">
+        <is>
+          <t>pending separate validated solution method</t>
+        </is>
+      </c>
+      <c r="R133" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S133" s="2" t="inlineStr">
+        <is>
+          <t>admissible under stated spin evidence</t>
+        </is>
+      </c>
+      <c r="T133" s="3" t="n">
         <v>-1.198326265264768</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T129"/>
+  <autoFilter ref="A1:T133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -49383,7 +50407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM26"/>
+  <dimension ref="A1:BM28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -55685,8 +56709,426 @@
         <v>0</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_ndi_ethyl</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>N-(4-methylbenzyl)-N-ethyl 1,2,3,4-naphthalene diimide</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>imide (n-type)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>gas UMA only</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_ndi_ethyl</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>CCn1c(=O)c2c3ccccc3c3c(=O)n(Cc4ccc(C)cc4)c(=O)c3c2c1=O</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>NANYKQXYZMYUQE-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>C24H18N2O4</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>CCn1c(=O)c2c3ccccc3c3c(=O)n([*:1])c(=O)c3c2c1=O</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>CCn1c(=O)c2c3ccccc3c3c(=O)[nH]c(=O)c3c2c1=O</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>[["neu", 0, 1, 0], ["red1", -1, 2, -1], ["red2", -2, 1, -2]]</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>verified exact-grafted graph/arithmetic</t>
+        </is>
+      </c>
+      <c r="P27" s="3" t="n">
+        <v>398.418</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R27" s="3" t="n">
+        <v>134.5</v>
+      </c>
+      <c r="S27" s="3" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="W27" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="X27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z27" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF27" s="2" t="inlineStr">
+        <is>
+          <t>partial/pending DFT spin validation</t>
+        </is>
+      </c>
+      <c r="AG27" s="2" t="n"/>
+      <c r="AH27" s="2" t="n"/>
+      <c r="AI27" s="2" t="n"/>
+      <c r="AJ27" s="2" t="n"/>
+      <c r="AK27" s="2" t="inlineStr">
+        <is>
+          <t>pending DFT spin validation</t>
+        </is>
+      </c>
+      <c r="AL27" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AM27" s="2" t="n"/>
+      <c r="AN27" s="2" t="n"/>
+      <c r="AO27" s="2" t="inlineStr">
+        <is>
+          <t>pending DFT spin validation</t>
+        </is>
+      </c>
+      <c r="AP27" s="2" t="n"/>
+      <c r="AQ27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS27" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3762/bjoc.20.155</t>
+        </is>
+      </c>
+      <c r="AT27" s="2" t="inlineStr">
+        <is>
+          <t>Test cata vs conventional NDI as a core-topology isomer pair with the same formula, ethyl cap and N-graft anchor. Source parents are bis-phenyl/bis-hexyl. Mixed N-ethyl/N-graft precursor isolation and selectivity are unverified. Parent measurements are in CH2Cl2 and are not exact-graft or MeCN labels.</t>
+        </is>
+      </c>
+      <c r="AU27" s="2" t="inlineStr">
+        <is>
+          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+        </is>
+      </c>
+      <c r="AV27" s="2" t="n"/>
+      <c r="AW27" s="2" t="n"/>
+      <c r="AX27" s="2" t="n"/>
+      <c r="AY27" s="2" t="n"/>
+      <c r="AZ27" s="2" t="n"/>
+      <c r="BA27" s="2" t="inlineStr">
+        <is>
+          <t>design_ndi_ethyl</t>
+        </is>
+      </c>
+      <c r="BB27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC27" s="2" t="inlineStr">
+        <is>
+          <t>DFT_check_required</t>
+        </is>
+      </c>
+      <c r="BD27" s="2" t="inlineStr">
+        <is>
+          <t>neu:UMA_large_gap_preliminary; red1:standard_doublet_model; red2:DFT_check_required</t>
+        </is>
+      </c>
+      <c r="BE27" s="2" t="n"/>
+      <c r="BF27" s="2" t="n"/>
+      <c r="BG27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH27" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI27" s="2" t="n"/>
+      <c r="BJ27" s="2" t="n"/>
+      <c r="BK27" s="2" t="n"/>
+      <c r="BL27" s="2" t="inlineStr">
+        <is>
+          <t>outside current queue</t>
+        </is>
+      </c>
+      <c r="BM27" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>N-(4-methylbenzyl)-N-ethyl 1,2,3,4-anthracene diimide</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>imide (n-type)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>gas UMA only</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>CCn1c(=O)c2c3cc4ccccc4cc3c3c(=O)n(Cc4ccc(C)cc4)c(=O)c3c2c1=O</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>LKTOOBTUSSFQCC-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>C28H20N2O4</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>CCn1c(=O)c2c3cc4ccccc4cc3c3c(=O)n([*:1])c(=O)c3c2c1=O</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>CCn1c(=O)c2c3cc4ccccc4cc3c3c(=O)[nH]c(=O)c3c2c1=O</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>[["neu", 0, 1, 0], ["red1", -1, 2, -1], ["red2", -2, 1, -2]]</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>verified exact-grafted graph/arithmetic</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="n">
+        <v>448.478</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R28" s="3" t="n">
+        <v>119.5</v>
+      </c>
+      <c r="S28" s="3" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="T28" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="W28" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="X28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z28" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF28" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AG28" s="2" t="n"/>
+      <c r="AH28" s="2" t="n"/>
+      <c r="AI28" s="2" t="n"/>
+      <c r="AJ28" s="2" t="n"/>
+      <c r="AK28" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AL28" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="AM28" s="2" t="n"/>
+      <c r="AN28" s="2" t="n"/>
+      <c r="AO28" s="2" t="inlineStr">
+        <is>
+          <t>pending electrolyte-window/integrity QC</t>
+        </is>
+      </c>
+      <c r="AP28" s="2" t="n"/>
+      <c r="AQ28" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR28" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS28" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3762/bjoc.20.155</t>
+        </is>
+      </c>
+      <c r="AT28" s="2" t="inlineStr">
+        <is>
+          <t>Test adding one fused benzene to the cata-NDI core, with the same ethyl cap and N-graft anchor; core size changes explicitly. Source parents are bis-phenyl/bis-hexyl. Mixed N-ethyl/N-graft precursor isolation and selectivity are unverified. Parent measurements are in CH2Cl2 and are not exact-graft or MeCN labels.</t>
+        </is>
+      </c>
+      <c r="AU28" s="2" t="inlineStr">
+        <is>
+          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+        </is>
+      </c>
+      <c r="AV28" s="2" t="n"/>
+      <c r="AW28" s="2" t="n"/>
+      <c r="AX28" s="2" t="n"/>
+      <c r="AY28" s="2" t="n"/>
+      <c r="AZ28" s="2" t="n"/>
+      <c r="BA28" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_ndi_ethyl</t>
+        </is>
+      </c>
+      <c r="BB28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC28" s="2" t="inlineStr">
+        <is>
+          <t>admissible stated spin model</t>
+        </is>
+      </c>
+      <c r="BD28" s="2" t="inlineStr">
+        <is>
+          <t>neu:UMA_large_gap_preliminary; red1:standard_doublet_model; red2:UMA_large_gap_preliminary</t>
+        </is>
+      </c>
+      <c r="BE28" s="2" t="n"/>
+      <c r="BF28" s="2" t="n"/>
+      <c r="BG28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH28" s="2" t="inlineStr">
+        <is>
+          <t>no_scoped_limitation</t>
+        </is>
+      </c>
+      <c r="BI28" s="2" t="n"/>
+      <c r="BJ28" s="2" t="n"/>
+      <c r="BK28" s="2" t="n"/>
+      <c r="BL28" s="2" t="inlineStr">
+        <is>
+          <t>outside current queue</t>
+        </is>
+      </c>
+      <c r="BM28" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:BM26"/>
+  <autoFilter ref="A1:BM28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -56321,7 +57763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -57270,8 +58712,58 @@
         <v>0</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_ndi_ethyl</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>design_ndi_ethyl</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>pending admitted event pair</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_adi_ethyl</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>hyp_cata_ndi_ethyl</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>pending admitted event pair</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I25"/>
+  <autoFilter ref="A1:I27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -57298,7 +58790,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-19T06:24:53.538237-05:00</t>
+          <t>2026-10-19T06:51:30.588734-05:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reproduce gas anchors and review cata derivative and spin corrections
</commit_message>
<xml_diff>
--- a/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
+++ b/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
@@ -38591,42 +38591,58 @@
         <v>0.01897270977497101</v>
       </c>
       <c r="P192" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q192" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R192" s="2" t="n"/>
-      <c r="S192" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T192" s="2" t="n"/>
-      <c r="U192" s="2" t="n"/>
-      <c r="V192" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q192" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R192" s="3" t="n">
+        <v>-36353.92114747687</v>
+      </c>
+      <c r="S192" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T192" s="3" t="n">
+        <v>8.596162152739655</v>
+      </c>
+      <c r="U192" s="3" t="n">
+        <v>8.596162152739655</v>
+      </c>
+      <c r="V192" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W192" s="2" t="n"/>
       <c r="X192" s="2" t="n"/>
-      <c r="Y192" s="2" t="n"/>
+      <c r="Y192" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z192" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA192" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB192" s="2" t="n"/>
-      <c r="AC192" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD192" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA192" s="2" t="inlineStr"/>
+      <c r="AB192" s="3" t="n">
+        <v>-36345.32498532413</v>
+      </c>
+      <c r="AC192" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD192" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/hyp_cata_ndi_ethyl/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE192" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_ndi_ethyl/neu/result.json</t>
@@ -38653,7 +38669,9 @@
       <c r="AJ192" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK192" s="2" t="n"/>
+      <c r="AK192" s="3" t="n">
+        <v>-36345.32498532413</v>
+      </c>
       <c r="AL192" s="2" t="n"/>
     </row>
     <row r="193">
@@ -38841,14 +38859,16 @@
         <v>0.01944873854517937</v>
       </c>
       <c r="P194" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q194" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R194" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q194" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R194" s="3" t="n">
+        <v>-36359.84626807191</v>
+      </c>
       <c r="S194" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -38856,10 +38876,18 @@
       </c>
       <c r="T194" s="2" t="n"/>
       <c r="U194" s="2" t="n"/>
-      <c r="V194" s="2" t="n"/>
+      <c r="V194" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W194" s="2" t="n"/>
       <c r="X194" s="2" t="n"/>
-      <c r="Y194" s="2" t="n"/>
+      <c r="Y194" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z194" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -38867,7 +38895,7 @@
       </c>
       <c r="AA194" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB194" s="2" t="n"/>
@@ -38876,7 +38904,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD194" s="2" t="n"/>
+      <c r="AD194" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/hyp_cata_ndi_ethyl/red2/result.json</t>
+        </is>
+      </c>
       <c r="AE194" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_ndi_ethyl/red2/result.json</t>
@@ -38967,14 +38999,16 @@
         <v>0.01762303523719311</v>
       </c>
       <c r="P195" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q195" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R195" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q195" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R195" s="3" t="n">
+        <v>-40534.65822548029</v>
+      </c>
       <c r="S195" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -38982,10 +39016,18 @@
       </c>
       <c r="T195" s="2" t="n"/>
       <c r="U195" s="2" t="n"/>
-      <c r="V195" s="2" t="n"/>
+      <c r="V195" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W195" s="2" t="n"/>
       <c r="X195" s="2" t="n"/>
-      <c r="Y195" s="2" t="n"/>
+      <c r="Y195" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z195" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -38993,7 +39035,7 @@
       </c>
       <c r="AA195" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB195" s="2" t="n"/>
@@ -39002,7 +39044,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD195" s="2" t="n"/>
+      <c r="AD195" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/hyp_cata_adi_ethyl/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE195" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_adi_ethyl/neu/result.json</t>
@@ -56729,7 +56775,7 @@
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>partial native surfaces; remaining states and spin validation pending</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -56814,16 +56860,16 @@
         <v>3</v>
       </c>
       <c r="AB27" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC27" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF27" s="2" t="inlineStr">
         <is>
@@ -56884,7 +56930,7 @@
         </is>
       </c>
       <c r="BB27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC27" s="2" t="inlineStr">
         <is>
@@ -56938,7 +56984,7 @@
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>active SP records present; native validation pending</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -57023,10 +57069,10 @@
         <v>3</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD28" s="2" t="n">
         <v>0</v>
@@ -58790,7 +58836,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-19T06:51:30.588734-05:00</t>
+          <t>2026-10-19T07:22:29.627012-05:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish both cata-imide ladders and the complete independently checked property tables
</commit_message>
<xml_diff>
--- a/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
+++ b/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
@@ -38735,42 +38735,58 @@
         <v>0.01764801330864429</v>
       </c>
       <c r="P193" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q193" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R193" s="2" t="n"/>
-      <c r="S193" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T193" s="2" t="n"/>
-      <c r="U193" s="2" t="n"/>
-      <c r="V193" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q193" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R193" s="3" t="n">
+        <v>-36357.23551539372</v>
+      </c>
+      <c r="S193" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T193" s="3" t="n">
+        <v>8.515316841382729</v>
+      </c>
+      <c r="U193" s="3" t="n">
+        <v>8.515316841382729</v>
+      </c>
+      <c r="V193" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W193" s="2" t="n"/>
       <c r="X193" s="2" t="n"/>
-      <c r="Y193" s="2" t="n"/>
+      <c r="Y193" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z193" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA193" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB193" s="2" t="n"/>
-      <c r="AC193" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD193" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA193" s="2" t="inlineStr"/>
+      <c r="AB193" s="3" t="n">
+        <v>-36348.72019855234</v>
+      </c>
+      <c r="AC193" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD193" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/hyp_cata_ndi_ethyl/red1/result.json</t>
+        </is>
+      </c>
       <c r="AE193" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_ndi_ethyl/red1/result.json</t>
@@ -38795,7 +38811,9 @@
       <c r="AJ193" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK193" s="2" t="n"/>
+      <c r="AK193" s="3" t="n">
+        <v>-36348.72019855234</v>
+      </c>
       <c r="AL193" s="2" t="n"/>
     </row>
     <row r="194">
@@ -38869,20 +38887,28 @@
       <c r="R194" s="3" t="n">
         <v>-36359.84626807191</v>
       </c>
-      <c r="S194" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T194" s="2" t="n"/>
-      <c r="U194" s="2" t="n"/>
+      <c r="S194" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T194" s="3" t="n">
+        <v>8.477071625259727</v>
+      </c>
+      <c r="U194" s="3" t="n">
+        <v>8.476967593173926</v>
+      </c>
       <c r="V194" s="2" t="inlineStr">
         <is>
-          <t>not_selected</t>
-        </is>
-      </c>
-      <c r="W194" s="2" t="n"/>
-      <c r="X194" s="2" t="n"/>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="W194" s="3" t="n">
+        <v>-0.0001040320858010091</v>
+      </c>
+      <c r="X194" s="3" t="n">
+        <v>0.004040923569666021</v>
+      </c>
       <c r="Y194" s="2" t="inlineStr">
         <is>
           <t>native_solution_dft_qrrho_spin</t>
@@ -38890,18 +38916,16 @@
       </c>
       <c r="Z194" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA194" s="2" t="inlineStr">
-        <is>
-          <t>missing_validated_native_thermal</t>
-        </is>
-      </c>
-      <c r="AB194" s="2" t="n"/>
-      <c r="AC194" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA194" s="2" t="inlineStr"/>
+      <c r="AB194" s="3" t="n">
+        <v>-36351.36930047873</v>
+      </c>
+      <c r="AC194" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
         </is>
       </c>
       <c r="AD194" s="2" t="inlineStr">
@@ -38916,27 +38940,31 @@
       </c>
       <c r="AF194" s="2" t="inlineStr">
         <is>
-          <t>DFT_check_required</t>
+          <t>DFT_native_equilibrium_ensemble</t>
         </is>
       </c>
       <c r="AG194" s="3" t="n">
-        <v>0.2348</v>
+        <v>0.1414950169346412</v>
       </c>
       <c r="AH194" s="2" t="inlineStr">
         <is>
-          <t>UMA gas preoptimization; solution ground state not independently established</t>
+          <t>two qualified native spin surfaces; equilibrium partition</t>
         </is>
       </c>
       <c r="AI194" s="2" t="inlineStr">
         <is>
-          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_ndi_ethyl/red2/result.json</t>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/hyp_cata_ndi_ethyl/red2/spin_ensemble_policy.json</t>
         </is>
       </c>
       <c r="AJ194" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK194" s="2" t="n"/>
-      <c r="AL194" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AK194" s="3" t="n">
+        <v>-36351.36930047873</v>
+      </c>
+      <c r="AL194" s="2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -39009,13 +39037,17 @@
       <c r="R195" s="3" t="n">
         <v>-40534.65822548029</v>
       </c>
-      <c r="S195" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T195" s="2" t="n"/>
-      <c r="U195" s="2" t="n"/>
+      <c r="S195" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T195" s="3" t="n">
+        <v>9.786087214095373</v>
+      </c>
+      <c r="U195" s="3" t="n">
+        <v>9.786087214095373</v>
+      </c>
       <c r="V195" s="2" t="inlineStr">
         <is>
           <t>not_selected</t>
@@ -39030,18 +39062,16 @@
       </c>
       <c r="Z195" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA195" s="2" t="inlineStr">
-        <is>
-          <t>missing_validated_native_thermal</t>
-        </is>
-      </c>
-      <c r="AB195" s="2" t="n"/>
-      <c r="AC195" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA195" s="2" t="inlineStr"/>
+      <c r="AB195" s="3" t="n">
+        <v>-40524.87213826619</v>
+      </c>
+      <c r="AC195" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
         </is>
       </c>
       <c r="AD195" s="2" t="inlineStr">
@@ -39075,7 +39105,9 @@
       <c r="AJ195" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK195" s="2" t="n"/>
+      <c r="AK195" s="3" t="n">
+        <v>-40524.87213826619</v>
+      </c>
       <c r="AL195" s="2" t="n"/>
     </row>
     <row r="196">
@@ -39139,42 +39171,58 @@
         <v>0.014229373075068</v>
       </c>
       <c r="P196" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q196" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R196" s="2" t="n"/>
-      <c r="S196" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T196" s="2" t="n"/>
-      <c r="U196" s="2" t="n"/>
-      <c r="V196" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q196" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R196" s="3" t="n">
+        <v>-40538.14948704982</v>
+      </c>
+      <c r="S196" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T196" s="3" t="n">
+        <v>9.709021130048876</v>
+      </c>
+      <c r="U196" s="3" t="n">
+        <v>9.709021130048876</v>
+      </c>
+      <c r="V196" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W196" s="2" t="n"/>
       <c r="X196" s="2" t="n"/>
-      <c r="Y196" s="2" t="n"/>
+      <c r="Y196" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z196" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA196" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB196" s="2" t="n"/>
-      <c r="AC196" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD196" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA196" s="2" t="inlineStr"/>
+      <c r="AB196" s="3" t="n">
+        <v>-40528.44046591978</v>
+      </c>
+      <c r="AC196" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD196" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/hyp_cata_adi_ethyl/red1/result.json</t>
+        </is>
+      </c>
       <c r="AE196" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_adi_ethyl/red1/result.json</t>
@@ -39199,7 +39247,9 @@
       <c r="AJ196" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK196" s="2" t="n"/>
+      <c r="AK196" s="3" t="n">
+        <v>-40528.44046591978</v>
+      </c>
       <c r="AL196" s="2" t="n"/>
     </row>
     <row r="197">
@@ -39263,42 +39313,58 @@
         <v>0.01947363466024399</v>
       </c>
       <c r="P197" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q197" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R197" s="2" t="n"/>
-      <c r="S197" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T197" s="2" t="n"/>
-      <c r="U197" s="2" t="n"/>
-      <c r="V197" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q197" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R197" s="3" t="n">
+        <v>-40540.97057035643</v>
+      </c>
+      <c r="S197" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T197" s="3" t="n">
+        <v>9.70153816634229</v>
+      </c>
+      <c r="U197" s="3" t="n">
+        <v>9.70153816634229</v>
+      </c>
+      <c r="V197" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W197" s="2" t="n"/>
       <c r="X197" s="2" t="n"/>
-      <c r="Y197" s="2" t="n"/>
+      <c r="Y197" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z197" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA197" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB197" s="2" t="n"/>
-      <c r="AC197" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD197" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA197" s="2" t="inlineStr"/>
+      <c r="AB197" s="3" t="n">
+        <v>-40531.26903219009</v>
+      </c>
+      <c r="AC197" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD197" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/hyp_cata_adi_ethyl/red2/result.json</t>
+        </is>
+      </c>
       <c r="AE197" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/hyp_cata_adi_ethyl/red2/result.json</t>
@@ -39325,7 +39391,9 @@
       <c r="AJ197" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK197" s="2" t="n"/>
+      <c r="AK197" s="3" t="n">
+        <v>-40531.26903219009</v>
+      </c>
       <c r="AL197" s="2" t="n"/>
     </row>
     <row r="198">
@@ -50039,25 +50107,37 @@
       <c r="F128" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="G128" s="2" t="n"/>
-      <c r="H128" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I128" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J128" s="2" t="n"/>
-      <c r="K128" s="2" t="n"/>
+      <c r="G128" s="3" t="n">
+        <v>-0.9839826733805239</v>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J128" s="3" t="n">
+        <v>3.314</v>
+      </c>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L128" s="2" t="n"/>
       <c r="M128" s="2" t="n"/>
-      <c r="N128" s="2" t="n"/>
-      <c r="O128" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="N128" s="2" t="inlineStr">
+        <is>
+          <t>conformer_jump</t>
+        </is>
+      </c>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>flagged diagnostic</t>
         </is>
       </c>
       <c r="P128" s="2" t="inlineStr">
@@ -50078,7 +50158,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="T128" s="2" t="n"/>
+      <c r="T128" s="3" t="n">
+        <v>-0.9839826733805239</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -50107,25 +50189,39 @@
       <c r="F129" s="2" t="n">
         <v>-2</v>
       </c>
-      <c r="G129" s="2" t="n"/>
+      <c r="G129" s="3" t="n">
+        <v>-1.73009397520218</v>
+      </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>pending DFT spin validation</t>
-        </is>
-      </c>
-      <c r="I129" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J129" s="2" t="n"/>
-      <c r="K129" s="2" t="n"/>
-      <c r="L129" s="2" t="n"/>
+          <t>native calculated/QC passed</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J129" s="3" t="n">
+        <v>2.611</v>
+      </c>
+      <c r="K129" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L129" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="M129" s="2" t="n"/>
-      <c r="N129" s="2" t="n"/>
-      <c r="O129" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="N129" s="2" t="inlineStr">
+        <is>
+          <t>anion_unbound+spin_ensemble_kinetics_unvalidated</t>
+        </is>
+      </c>
+      <c r="O129" s="2" t="inlineStr">
+        <is>
+          <t>flagged diagnostic</t>
         </is>
       </c>
       <c r="P129" s="2" t="inlineStr">
@@ -50143,10 +50239,12 @@
       </c>
       <c r="S129" s="2" t="inlineStr">
         <is>
-          <t>DFT spin validation required/wrong ground state</t>
-        </is>
-      </c>
-      <c r="T129" s="2" t="n"/>
+          <t>admissible under stated spin evidence</t>
+        </is>
+      </c>
+      <c r="T129" s="3" t="n">
+        <v>-1.73009397520218</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -50175,25 +50273,37 @@
       <c r="F130" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="G130" s="2" t="n"/>
-      <c r="H130" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I130" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J130" s="2" t="n"/>
-      <c r="K130" s="2" t="n"/>
+      <c r="G130" s="3" t="n">
+        <v>-0.8108682480087737</v>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J130" s="3" t="n">
+        <v>3.491</v>
+      </c>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L130" s="2" t="n"/>
       <c r="M130" s="2" t="n"/>
-      <c r="N130" s="2" t="n"/>
-      <c r="O130" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="N130" s="2" t="inlineStr">
+        <is>
+          <t>conformer_jump</t>
+        </is>
+      </c>
+      <c r="O130" s="2" t="inlineStr">
+        <is>
+          <t>flagged diagnostic</t>
         </is>
       </c>
       <c r="P130" s="2" t="inlineStr">
@@ -50214,7 +50324,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="T130" s="2" t="n"/>
+      <c r="T130" s="3" t="n">
+        <v>-0.8108682480087737</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -50243,25 +50355,37 @@
       <c r="F131" s="2" t="n">
         <v>-2</v>
       </c>
-      <c r="G131" s="2" t="n"/>
-      <c r="H131" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I131" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J131" s="2" t="n"/>
-      <c r="K131" s="2" t="n"/>
+      <c r="G131" s="3" t="n">
+        <v>-1.550629631281481</v>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J131" s="3" t="n">
+        <v>2.821</v>
+      </c>
+      <c r="K131" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L131" s="2" t="n"/>
       <c r="M131" s="2" t="n"/>
-      <c r="N131" s="2" t="n"/>
-      <c r="O131" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="N131" s="2" t="inlineStr">
+        <is>
+          <t>anion_unbound</t>
+        </is>
+      </c>
+      <c r="O131" s="2" t="inlineStr">
+        <is>
+          <t>flagged diagnostic</t>
         </is>
       </c>
       <c r="P131" s="2" t="inlineStr">
@@ -50282,7 +50406,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="T131" s="2" t="n"/>
+      <c r="T131" s="3" t="n">
+        <v>-1.550629631281481</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -56775,7 +56901,7 @@
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>partial native surfaces; remaining states and spin validation pending</t>
+          <t>native solution states complete</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -56860,44 +56986,54 @@
         <v>3</v>
       </c>
       <c r="AB27" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC27" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD27" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE27" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AF27" s="2" t="inlineStr">
         <is>
-          <t>partial/pending DFT spin validation</t>
-        </is>
-      </c>
-      <c r="AG27" s="2" t="n"/>
-      <c r="AH27" s="2" t="n"/>
-      <c r="AI27" s="2" t="n"/>
-      <c r="AJ27" s="2" t="n"/>
+          <t>verified native calculation</t>
+        </is>
+      </c>
+      <c r="AG27" s="3" t="n">
+        <v>-0.9839826733805239</v>
+      </c>
+      <c r="AH27" s="3" t="n">
+        <v>-1.73009397520218</v>
+      </c>
+      <c r="AI27" s="3" t="n">
+        <v>0.7461113018216565</v>
+      </c>
+      <c r="AJ27" s="3" t="n">
+        <v>71.98879675474809</v>
+      </c>
       <c r="AK27" s="2" t="inlineStr">
         <is>
-          <t>pending DFT spin validation</t>
-        </is>
-      </c>
-      <c r="AL27" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+          <t>native thermodynamic calculation; decomposition untested</t>
+        </is>
+      </c>
+      <c r="AL27" s="2" t="inlineStr">
+        <is>
+          <t>gas diagnostic available; solution descriptor pending</t>
         </is>
       </c>
       <c r="AM27" s="2" t="n"/>
       <c r="AN27" s="2" t="n"/>
       <c r="AO27" s="2" t="inlineStr">
         <is>
-          <t>pending DFT spin validation</t>
-        </is>
-      </c>
-      <c r="AP27" s="2" t="n"/>
+          <t>computed native-window/integrity bookkeeping; kinetic QC separate</t>
+        </is>
+      </c>
+      <c r="AP27" s="3" t="n">
+        <v>134.5395094822244</v>
+      </c>
       <c r="AQ27" s="2" t="b">
         <v>0</v>
       </c>
@@ -56916,7 +57052,7 @@
       </c>
       <c r="AU27" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV27" s="2" t="n"/>
@@ -56930,20 +57066,24 @@
         </is>
       </c>
       <c r="BB27" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BC27" s="2" t="inlineStr">
         <is>
-          <t>DFT_check_required</t>
+          <t>admissible stated spin model</t>
         </is>
       </c>
       <c r="BD27" s="2" t="inlineStr">
         <is>
-          <t>neu:UMA_large_gap_preliminary; red1:standard_doublet_model; red2:DFT_check_required</t>
-        </is>
-      </c>
-      <c r="BE27" s="2" t="n"/>
-      <c r="BF27" s="2" t="n"/>
+          <t>neu:UMA_large_gap_preliminary; red1:standard_doublet_model; red2:DFT_native_equilibrium_ensemble</t>
+        </is>
+      </c>
+      <c r="BE27" s="3" t="n">
+        <v>-0.9839826733805239</v>
+      </c>
+      <c r="BF27" s="3" t="n">
+        <v>-1.73009397520218</v>
+      </c>
       <c r="BG27" s="2" t="b">
         <v>1</v>
       </c>
@@ -56954,7 +57094,9 @@
       </c>
       <c r="BI27" s="2" t="n"/>
       <c r="BJ27" s="2" t="n"/>
-      <c r="BK27" s="2" t="n"/>
+      <c r="BK27" s="3" t="n">
+        <v>134.5395094822244</v>
+      </c>
       <c r="BL27" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
@@ -56984,7 +57126,7 @@
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>active SP records present; native validation pending</t>
+          <t>native solution states complete</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -57069,44 +57211,54 @@
         <v>3</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AD28" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AE28" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF28" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AG28" s="2" t="n"/>
-      <c r="AH28" s="2" t="n"/>
-      <c r="AI28" s="2" t="n"/>
-      <c r="AJ28" s="2" t="n"/>
-      <c r="AK28" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AL28" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+        <v>3</v>
+      </c>
+      <c r="AF28" s="2" t="inlineStr">
+        <is>
+          <t>verified native calculation</t>
+        </is>
+      </c>
+      <c r="AG28" s="3" t="n">
+        <v>-0.8108682480087737</v>
+      </c>
+      <c r="AH28" s="3" t="n">
+        <v>-1.550629631281481</v>
+      </c>
+      <c r="AI28" s="3" t="n">
+        <v>0.7397613832727075</v>
+      </c>
+      <c r="AJ28" s="3" t="n">
+        <v>71.3761227546178</v>
+      </c>
+      <c r="AK28" s="2" t="inlineStr">
+        <is>
+          <t>native thermodynamic calculation; decomposition untested</t>
+        </is>
+      </c>
+      <c r="AL28" s="2" t="inlineStr">
+        <is>
+          <t>gas diagnostic available; solution descriptor pending</t>
         </is>
       </c>
       <c r="AM28" s="2" t="n"/>
       <c r="AN28" s="2" t="n"/>
       <c r="AO28" s="2" t="inlineStr">
         <is>
-          <t>pending electrolyte-window/integrity QC</t>
-        </is>
-      </c>
-      <c r="AP28" s="2" t="n"/>
+          <t>computed native-window/integrity bookkeeping; kinetic QC separate</t>
+        </is>
+      </c>
+      <c r="AP28" s="3" t="n">
+        <v>119.5219437495014</v>
+      </c>
       <c r="AQ28" s="2" t="b">
         <v>0</v>
       </c>
@@ -57125,7 +57277,7 @@
       </c>
       <c r="AU28" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV28" s="2" t="n"/>
@@ -57139,7 +57291,7 @@
         </is>
       </c>
       <c r="BB28" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BC28" s="2" t="inlineStr">
         <is>
@@ -57151,8 +57303,12 @@
           <t>neu:UMA_large_gap_preliminary; red1:standard_doublet_model; red2:UMA_large_gap_preliminary</t>
         </is>
       </c>
-      <c r="BE28" s="2" t="n"/>
-      <c r="BF28" s="2" t="n"/>
+      <c r="BE28" s="3" t="n">
+        <v>-0.8108682480087737</v>
+      </c>
+      <c r="BF28" s="3" t="n">
+        <v>-1.550629631281481</v>
+      </c>
       <c r="BG28" s="2" t="b">
         <v>1</v>
       </c>
@@ -57163,7 +57319,9 @@
       </c>
       <c r="BI28" s="2" t="n"/>
       <c r="BJ28" s="2" t="n"/>
-      <c r="BK28" s="2" t="n"/>
+      <c r="BK28" s="3" t="n">
+        <v>119.5219437495014</v>
+      </c>
       <c r="BL28" s="2" t="inlineStr">
         <is>
           <t>outside current queue</t>
@@ -58771,12 +58929,18 @@
           <t>design_ndi_ethyl</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
+      <c r="E26" s="3" t="n">
+        <v>-0.2199670601330581</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>-0.3116112859643181</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>0.09164422583125997</v>
+      </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>pending admitted event pair</t>
+          <t>both potential shifts admitted</t>
         </is>
       </c>
       <c r="I26" s="2" t="b">
@@ -58796,12 +58960,18 @@
           <t>hyp_cata_ndi_ethyl</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
+      <c r="E27" s="3" t="n">
+        <v>0.1731144253717503</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>0.1794643439206993</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>-0.006349918548949063</v>
+      </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>pending admitted event pair</t>
+          <t>both potential shifts admitted</t>
         </is>
       </c>
       <c r="I27" s="2" t="b">
@@ -58836,7 +59006,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-19T07:22:29.627012-05:00</t>
+          <t>2026-10-19T08:36:40.054609-05:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preserve aryl stages during H100 recovery and start distinct hexyl basins
Independently review five native states (303 checks), refresh the stable candidate export (613 checks), and rebuild the checked slide PDF. Route aryl memory failures to reserved H100s with byte-preserved stage resumption, sealed owner-release proofs and bounded attempts. Verify the first actual H100 native-stage resume and two isolated hexyl optimizer starts. Retain one separate Hessian symmetry hold and pending exact-graft properties. Full shared-workspace suite: 572 passing tests. Preserve concurrent exporter/plotting work and unrelated staged archive changes; retain the exact exporter source used for the checked snapshot as evidence.
</commit_message>
<xml_diff>
--- a/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
+++ b/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
@@ -39457,14 +39457,16 @@
         <v>0.01970009692013264</v>
       </c>
       <c r="P198" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q198" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R198" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q198" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R198" s="3" t="n">
+        <v>-44770.23269187962</v>
+      </c>
       <c r="S198" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -39472,10 +39474,18 @@
       </c>
       <c r="T198" s="2" t="n"/>
       <c r="U198" s="2" t="n"/>
-      <c r="V198" s="2" t="n"/>
+      <c r="V198" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W198" s="2" t="n"/>
       <c r="X198" s="2" t="n"/>
-      <c r="Y198" s="2" t="n"/>
+      <c r="Y198" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z198" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -39483,7 +39493,7 @@
       </c>
       <c r="AA198" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB198" s="2" t="n"/>
@@ -39492,7 +39502,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD198" s="2" t="n"/>
+      <c r="AD198" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_0d7aa75989e9/ox2/result.json</t>
+        </is>
+      </c>
       <c r="AE198" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_0d7aa75989e9/ox2/result.json</t>
@@ -39707,14 +39721,16 @@
         <v>0.01833751983940601</v>
       </c>
       <c r="P200" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q200" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R200" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q200" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R200" s="3" t="n">
+        <v>-44777.50685478656</v>
+      </c>
       <c r="S200" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -39722,10 +39738,18 @@
       </c>
       <c r="T200" s="2" t="n"/>
       <c r="U200" s="2" t="n"/>
-      <c r="V200" s="2" t="n"/>
+      <c r="V200" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W200" s="2" t="n"/>
       <c r="X200" s="2" t="n"/>
-      <c r="Y200" s="2" t="n"/>
+      <c r="Y200" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z200" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -39733,7 +39757,7 @@
       </c>
       <c r="AA200" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB200" s="2" t="n"/>
@@ -39742,7 +39766,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD200" s="2" t="n"/>
+      <c r="AD200" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_0d7aa75989e9/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE200" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_0d7aa75989e9/neu/result.json</t>
@@ -39833,14 +39861,16 @@
         <v>0.01974492706358433</v>
       </c>
       <c r="P201" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q201" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R201" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q201" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R201" s="3" t="n">
+        <v>-44770.22165023634</v>
+      </c>
       <c r="S201" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -39848,10 +39878,18 @@
       </c>
       <c r="T201" s="2" t="n"/>
       <c r="U201" s="2" t="n"/>
-      <c r="V201" s="2" t="n"/>
+      <c r="V201" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W201" s="2" t="n"/>
       <c r="X201" s="2" t="n"/>
-      <c r="Y201" s="2" t="n"/>
+      <c r="Y201" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z201" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -39859,7 +39897,7 @@
       </c>
       <c r="AA201" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB201" s="2" t="n"/>
@@ -39868,7 +39906,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD201" s="2" t="n"/>
+      <c r="AD201" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_45a6c406cdc7/ox2/result.json</t>
+        </is>
+      </c>
       <c r="AE201" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_45a6c406cdc7/ox2/result.json</t>
@@ -40083,14 +40125,16 @@
         <v>0.01765217632055283</v>
       </c>
       <c r="P203" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q203" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R203" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q203" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R203" s="3" t="n">
+        <v>-44777.59741793967</v>
+      </c>
       <c r="S203" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -40098,10 +40142,18 @@
       </c>
       <c r="T203" s="2" t="n"/>
       <c r="U203" s="2" t="n"/>
-      <c r="V203" s="2" t="n"/>
+      <c r="V203" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W203" s="2" t="n"/>
       <c r="X203" s="2" t="n"/>
-      <c r="Y203" s="2" t="n"/>
+      <c r="Y203" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z203" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -40109,7 +40161,7 @@
       </c>
       <c r="AA203" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB203" s="2" t="n"/>
@@ -40118,7 +40170,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD203" s="2" t="n"/>
+      <c r="AD203" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_45a6c406cdc7/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE203" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_45a6c406cdc7/neu/result.json</t>
@@ -40711,14 +40767,16 @@
         <v>0.01966086402535439</v>
       </c>
       <c r="P208" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q208" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R208" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q208" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R208" s="3" t="n">
+        <v>-55039.26412296712</v>
+      </c>
       <c r="S208" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -40726,10 +40784,18 @@
       </c>
       <c r="T208" s="2" t="n"/>
       <c r="U208" s="2" t="n"/>
-      <c r="V208" s="2" t="n"/>
+      <c r="V208" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W208" s="2" t="n"/>
       <c r="X208" s="2" t="n"/>
-      <c r="Y208" s="2" t="n"/>
+      <c r="Y208" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z208" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -40737,7 +40803,7 @@
       </c>
       <c r="AA208" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB208" s="2" t="n"/>
@@ -40746,7 +40812,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD208" s="2" t="n"/>
+      <c r="AD208" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_4602f4a856c7/ox1/result.json</t>
+        </is>
+      </c>
       <c r="AE208" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_4602f4a856c7/ox1/result.json</t>
@@ -40835,42 +40905,58 @@
         <v>0.01952131278812885</v>
       </c>
       <c r="P209" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q209" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R209" s="2" t="n"/>
-      <c r="S209" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T209" s="2" t="n"/>
-      <c r="U209" s="2" t="n"/>
-      <c r="V209" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q209" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R209" s="3" t="n">
+        <v>-55042.76098553109</v>
+      </c>
+      <c r="S209" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T209" s="3" t="n">
+        <v>12.72804878583608</v>
+      </c>
+      <c r="U209" s="3" t="n">
+        <v>12.72804878583608</v>
+      </c>
+      <c r="V209" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W209" s="2" t="n"/>
       <c r="X209" s="2" t="n"/>
-      <c r="Y209" s="2" t="n"/>
+      <c r="Y209" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z209" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA209" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB209" s="2" t="n"/>
-      <c r="AC209" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD209" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA209" s="2" t="inlineStr"/>
+      <c r="AB209" s="3" t="n">
+        <v>-55030.03293674526</v>
+      </c>
+      <c r="AC209" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD209" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_4602f4a856c7/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE209" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_4602f4a856c7/neu/result.json</t>
@@ -40897,7 +40983,9 @@
       <c r="AJ209" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK209" s="2" t="n"/>
+      <c r="AK209" s="3" t="n">
+        <v>-55030.03293674526</v>
+      </c>
       <c r="AL209" s="2" t="n"/>
     </row>
     <row r="210">
@@ -40961,42 +41049,58 @@
         <v>0.01875787600874901</v>
       </c>
       <c r="P210" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q210" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R210" s="2" t="n"/>
-      <c r="S210" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T210" s="2" t="n"/>
-      <c r="U210" s="2" t="n"/>
-      <c r="V210" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q210" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R210" s="3" t="n">
+        <v>-55035.29337477739</v>
+      </c>
+      <c r="S210" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T210" s="3" t="n">
+        <v>12.84598680221423</v>
+      </c>
+      <c r="U210" s="3" t="n">
+        <v>12.84598680221423</v>
+      </c>
+      <c r="V210" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W210" s="2" t="n"/>
       <c r="X210" s="2" t="n"/>
-      <c r="Y210" s="2" t="n"/>
+      <c r="Y210" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z210" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA210" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB210" s="2" t="n"/>
-      <c r="AC210" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD210" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA210" s="2" t="inlineStr"/>
+      <c r="AB210" s="3" t="n">
+        <v>-55022.44738797517</v>
+      </c>
+      <c r="AC210" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD210" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_e2795f06393d/ox2/result.json</t>
+        </is>
+      </c>
       <c r="AE210" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_e2795f06393d/ox2/result.json</t>
@@ -41023,7 +41127,9 @@
       <c r="AJ210" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK210" s="2" t="n"/>
+      <c r="AK210" s="3" t="n">
+        <v>-55022.44738797517</v>
+      </c>
       <c r="AL210" s="2" t="n"/>
     </row>
     <row r="211">
@@ -41087,14 +41193,16 @@
         <v>0.01691009663045406</v>
       </c>
       <c r="P211" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q211" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R211" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q211" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R211" s="3" t="n">
+        <v>-55039.23756179307</v>
+      </c>
       <c r="S211" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -41102,10 +41210,18 @@
       </c>
       <c r="T211" s="2" t="n"/>
       <c r="U211" s="2" t="n"/>
-      <c r="V211" s="2" t="n"/>
+      <c r="V211" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W211" s="2" t="n"/>
       <c r="X211" s="2" t="n"/>
-      <c r="Y211" s="2" t="n"/>
+      <c r="Y211" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z211" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -41113,7 +41229,7 @@
       </c>
       <c r="AA211" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB211" s="2" t="n"/>
@@ -41122,7 +41238,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD211" s="2" t="n"/>
+      <c r="AD211" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_e2795f06393d/ox1/result.json</t>
+        </is>
+      </c>
       <c r="AE211" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_e2795f06393d/ox1/result.json</t>
@@ -41211,42 +41331,58 @@
         <v>0.01913126930594444</v>
       </c>
       <c r="P212" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q212" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R212" s="2" t="n"/>
-      <c r="S212" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T212" s="2" t="n"/>
-      <c r="U212" s="2" t="n"/>
-      <c r="V212" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q212" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R212" s="3" t="n">
+        <v>-55042.7173099153</v>
+      </c>
+      <c r="S212" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T212" s="3" t="n">
+        <v>12.73299806206877</v>
+      </c>
+      <c r="U212" s="3" t="n">
+        <v>12.73299806206877</v>
+      </c>
+      <c r="V212" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W212" s="2" t="n"/>
       <c r="X212" s="2" t="n"/>
-      <c r="Y212" s="2" t="n"/>
+      <c r="Y212" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z212" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA212" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB212" s="2" t="n"/>
-      <c r="AC212" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD212" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA212" s="2" t="inlineStr"/>
+      <c r="AB212" s="3" t="n">
+        <v>-55029.98431185323</v>
+      </c>
+      <c r="AC212" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD212" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_e2795f06393d/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE212" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_e2795f06393d/neu/result.json</t>
@@ -41273,7 +41409,9 @@
       <c r="AJ212" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK212" s="2" t="n"/>
+      <c r="AK212" s="3" t="n">
+        <v>-55029.98431185323</v>
+      </c>
       <c r="AL212" s="2" t="n"/>
     </row>
     <row r="213">
@@ -41337,42 +41475,58 @@
         <v>0.01962669938802719</v>
       </c>
       <c r="P213" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q213" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R213" s="2" t="n"/>
-      <c r="S213" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T213" s="2" t="n"/>
-      <c r="U213" s="2" t="n"/>
-      <c r="V213" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q213" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R213" s="3" t="n">
+        <v>-55035.39535531749</v>
+      </c>
+      <c r="S213" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T213" s="3" t="n">
+        <v>12.91432768474093</v>
+      </c>
+      <c r="U213" s="3" t="n">
+        <v>12.91432768474093</v>
+      </c>
+      <c r="V213" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W213" s="2" t="n"/>
       <c r="X213" s="2" t="n"/>
-      <c r="Y213" s="2" t="n"/>
+      <c r="Y213" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z213" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA213" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB213" s="2" t="n"/>
-      <c r="AC213" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD213" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA213" s="2" t="inlineStr"/>
+      <c r="AB213" s="3" t="n">
+        <v>-55022.48102763275</v>
+      </c>
+      <c r="AC213" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD213" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_c88a8d5645d4/ox2/result.json</t>
+        </is>
+      </c>
       <c r="AE213" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_c88a8d5645d4/ox2/result.json</t>
@@ -41399,7 +41553,9 @@
       <c r="AJ213" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK213" s="2" t="n"/>
+      <c r="AK213" s="3" t="n">
+        <v>-55022.48102763275</v>
+      </c>
       <c r="AL213" s="2" t="n"/>
     </row>
     <row r="214">
@@ -41587,42 +41743,58 @@
         <v>0.01976482942700386</v>
       </c>
       <c r="P215" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q215" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R215" s="2" t="n"/>
-      <c r="S215" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T215" s="2" t="n"/>
-      <c r="U215" s="2" t="n"/>
-      <c r="V215" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q215" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R215" s="3" t="n">
+        <v>-55042.67923586673</v>
+      </c>
+      <c r="S215" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T215" s="3" t="n">
+        <v>12.76147126871538</v>
+      </c>
+      <c r="U215" s="3" t="n">
+        <v>12.76147126871538</v>
+      </c>
+      <c r="V215" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W215" s="2" t="n"/>
       <c r="X215" s="2" t="n"/>
-      <c r="Y215" s="2" t="n"/>
+      <c r="Y215" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z215" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA215" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB215" s="2" t="n"/>
-      <c r="AC215" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD215" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA215" s="2" t="inlineStr"/>
+      <c r="AB215" s="3" t="n">
+        <v>-55029.91776459802</v>
+      </c>
+      <c r="AC215" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD215" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_c88a8d5645d4/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE215" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_c88a8d5645d4/neu/result.json</t>
@@ -41649,7 +41821,9 @@
       <c r="AJ215" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK215" s="2" t="n"/>
+      <c r="AK215" s="3" t="n">
+        <v>-55029.91776459802</v>
+      </c>
       <c r="AL215" s="2" t="n"/>
     </row>
     <row r="216">
@@ -42089,14 +42263,16 @@
         <v>0.01944122090935707</v>
       </c>
       <c r="P219" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q219" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R219" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q219" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R219" s="3" t="n">
+        <v>-42694.79467073609</v>
+      </c>
       <c r="S219" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -42104,10 +42280,18 @@
       </c>
       <c r="T219" s="2" t="n"/>
       <c r="U219" s="2" t="n"/>
-      <c r="V219" s="2" t="n"/>
+      <c r="V219" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W219" s="2" t="n"/>
       <c r="X219" s="2" t="n"/>
-      <c r="Y219" s="2" t="n"/>
+      <c r="Y219" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z219" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -42115,7 +42299,7 @@
       </c>
       <c r="AA219" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB219" s="2" t="n"/>
@@ -42124,7 +42308,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD219" s="2" t="n"/>
+      <c r="AD219" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_9992bd3479e1/ox2/result.json</t>
+        </is>
+      </c>
       <c r="AE219" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_9992bd3479e1/ox2/result.json</t>
@@ -54303,13 +54491,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I139" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J139" s="2" t="n"/>
-      <c r="K139" s="2" t="n"/>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J139" s="3" t="n">
+        <v>3.497</v>
+      </c>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L139" s="2" t="n"/>
       <c r="M139" s="2" t="n"/>
       <c r="N139" s="2" t="n"/>
@@ -54371,13 +54565,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I140" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J140" s="2" t="n"/>
-      <c r="K140" s="2" t="n"/>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J140" s="3" t="n">
+        <v>3.944</v>
+      </c>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L140" s="2" t="n"/>
       <c r="M140" s="2" t="n"/>
       <c r="N140" s="2" t="n"/>
@@ -54439,13 +54639,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I141" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J141" s="2" t="n"/>
-      <c r="K141" s="2" t="n"/>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J141" s="3" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L141" s="2" t="n"/>
       <c r="M141" s="2" t="n"/>
       <c r="N141" s="2" t="n"/>
@@ -61959,7 +62165,7 @@
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>active SP records present; native validation pending</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -62044,10 +62250,10 @@
         <v>3</v>
       </c>
       <c r="AB29" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC29" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD29" s="2" t="n">
         <v>0</v>
@@ -62133,7 +62339,7 @@
       <c r="BK29" s="2" t="n"/>
       <c r="BL29" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 3 producer reports in progress; 0 queued/unresolved; field-specific QC separate</t>
+          <t>0/3 surface records verified; 2 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 1 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM29" s="2" t="b">
@@ -62160,7 +62366,7 @@
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>active SP records present; native validation pending</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -62245,10 +62451,10 @@
         <v>3</v>
       </c>
       <c r="AB30" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD30" s="2" t="n">
         <v>0</v>
@@ -62334,7 +62540,7 @@
       <c r="BK30" s="2" t="n"/>
       <c r="BL30" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 3 producer reports in progress; 0 queued/unresolved; field-specific QC separate</t>
+          <t>0/3 surface records verified; 3 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM30" s="2" t="b">
@@ -62535,7 +62741,7 @@
       <c r="BK31" s="2" t="n"/>
       <c r="BL31" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 3 producer reports in progress; 0 queued/unresolved; field-specific QC separate</t>
+          <t>0/3 surface records verified; 2 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 1 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM31" s="2" t="b">
@@ -62562,7 +62768,7 @@
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>partial native solution states; remaining states pending</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -62647,16 +62853,16 @@
         <v>3</v>
       </c>
       <c r="AB32" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD32" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE32" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF32" s="4" t="inlineStr">
         <is>
@@ -62709,7 +62915,7 @@
       <c r="AZ32" s="2" t="n"/>
       <c r="BA32" s="2" t="n"/>
       <c r="BB32" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC32" s="2" t="inlineStr">
         <is>
@@ -62736,7 +62942,7 @@
       <c r="BK32" s="2" t="n"/>
       <c r="BL32" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 3 producer reports in progress; 0 queued/unresolved; field-specific QC separate</t>
+          <t>1/3 surface records verified; 1 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM32" s="2" t="b">
@@ -62763,7 +62969,7 @@
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>partial native solution states; remaining states pending</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -62848,16 +63054,16 @@
         <v>3</v>
       </c>
       <c r="AB33" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC33" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD33" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE33" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF33" s="4" t="inlineStr">
         <is>
@@ -62900,7 +63106,7 @@
       </c>
       <c r="AU33" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV33" s="2" t="n"/>
@@ -62910,7 +63116,7 @@
       <c r="AZ33" s="2" t="n"/>
       <c r="BA33" s="2" t="n"/>
       <c r="BB33" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BC33" s="2" t="inlineStr">
         <is>
@@ -62937,7 +63143,7 @@
       <c r="BK33" s="2" t="n"/>
       <c r="BL33" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 3 producer reports in progress; 0 queued/unresolved; field-specific QC separate</t>
+          <t>2/3 surface records verified; 0 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM33" s="2" t="b">
@@ -62964,7 +63170,7 @@
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>partial native solution states; remaining states pending</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -63049,16 +63255,16 @@
         <v>3</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD34" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE34" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF34" s="4" t="inlineStr">
         <is>
@@ -63111,7 +63317,7 @@
       <c r="AZ34" s="2" t="n"/>
       <c r="BA34" s="2" t="n"/>
       <c r="BB34" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BC34" s="2" t="inlineStr">
         <is>
@@ -63138,7 +63344,7 @@
       <c r="BK34" s="2" t="n"/>
       <c r="BL34" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 3 producer reports in progress; 0 queued/unresolved; field-specific QC separate</t>
+          <t>2/3 surface records verified; 0 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM34" s="2" t="b">
@@ -63339,7 +63545,7 @@
       <c r="BK35" s="2" t="n"/>
       <c r="BL35" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 0 producer reports in progress; 3 queued/unresolved; field-specific QC separate</t>
+          <t>0/3 surface records verified; 0 failed/preserved; 3 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM35" s="2" t="b">
@@ -63366,7 +63572,7 @@
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>active SP records present; native validation pending</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -63451,10 +63657,10 @@
         <v>3</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD36" s="2" t="n">
         <v>0</v>
@@ -63540,7 +63746,7 @@
       <c r="BK36" s="2" t="n"/>
       <c r="BL36" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 0 producer reports in progress; 3 queued/unresolved; field-specific QC separate</t>
+          <t>0/3 surface records verified; 0 failed/preserved; 2 producer reports in progress; 0 queued/unresolved; 1 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM36" s="2" t="b">
@@ -63741,7 +63947,7 @@
       <c r="BK37" s="2" t="n"/>
       <c r="BL37" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 0 producer reports in progress; 3 queued/unresolved; field-specific QC separate</t>
+          <t>0/3 surface records verified; 2 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 1 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM37" s="2" t="b">
@@ -65423,7 +65629,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-19T11:34:39.450415-05:00</t>
+          <t>2026-10-19T12:22:05.478576-05:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Organize maintained candidate figures and preserve working publication links
</commit_message>
<xml_diff>
--- a/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
+++ b/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
@@ -39597,14 +39597,16 @@
         <v>0.01962625049054623</v>
       </c>
       <c r="P199" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q199" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R199" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q199" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R199" s="3" t="n">
+        <v>-44774.12778660435</v>
+      </c>
       <c r="S199" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -39612,10 +39614,18 @@
       </c>
       <c r="T199" s="2" t="n"/>
       <c r="U199" s="2" t="n"/>
-      <c r="V199" s="2" t="n"/>
+      <c r="V199" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W199" s="2" t="n"/>
       <c r="X199" s="2" t="n"/>
-      <c r="Y199" s="2" t="n"/>
+      <c r="Y199" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z199" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -39623,7 +39633,7 @@
       </c>
       <c r="AA199" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB199" s="2" t="n"/>
@@ -39632,7 +39642,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD199" s="2" t="n"/>
+      <c r="AD199" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_0d7aa75989e9/ox1/result.json</t>
+        </is>
+      </c>
       <c r="AE199" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_0d7aa75989e9/ox1/result.json</t>
@@ -40001,14 +40015,16 @@
         <v>0.01543018128722906</v>
       </c>
       <c r="P202" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q202" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R202" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q202" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R202" s="3" t="n">
+        <v>-44774.14750819249</v>
+      </c>
       <c r="S202" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -40016,10 +40032,18 @@
       </c>
       <c r="T202" s="2" t="n"/>
       <c r="U202" s="2" t="n"/>
-      <c r="V202" s="2" t="n"/>
+      <c r="V202" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W202" s="2" t="n"/>
       <c r="X202" s="2" t="n"/>
-      <c r="Y202" s="2" t="n"/>
+      <c r="Y202" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z202" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -40027,7 +40051,7 @@
       </c>
       <c r="AA202" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB202" s="2" t="n"/>
@@ -40036,7 +40060,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD202" s="2" t="n"/>
+      <c r="AD202" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_45a6c406cdc7/ox1/result.json</t>
+        </is>
+      </c>
       <c r="AE202" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_45a6c406cdc7/ox1/result.json</t>
@@ -40265,42 +40293,58 @@
         <v>0.01968466117978096</v>
       </c>
       <c r="P204" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q204" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R204" s="2" t="n"/>
-      <c r="S204" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T204" s="2" t="n"/>
-      <c r="U204" s="2" t="n"/>
-      <c r="V204" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q204" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R204" s="3" t="n">
+        <v>-55035.63973132632</v>
+      </c>
+      <c r="S204" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T204" s="3" t="n">
+        <v>12.83295569022984</v>
+      </c>
+      <c r="U204" s="3" t="n">
+        <v>12.83295569022984</v>
+      </c>
+      <c r="V204" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W204" s="2" t="n"/>
       <c r="X204" s="2" t="n"/>
-      <c r="Y204" s="2" t="n"/>
+      <c r="Y204" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z204" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA204" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB204" s="2" t="n"/>
-      <c r="AC204" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD204" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA204" s="2" t="inlineStr"/>
+      <c r="AB204" s="3" t="n">
+        <v>-55022.80677563608</v>
+      </c>
+      <c r="AC204" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD204" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_c285539322fa/ox2/result.json</t>
+        </is>
+      </c>
       <c r="AE204" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_c285539322fa/ox2/result.json</t>
@@ -40327,7 +40371,9 @@
       <c r="AJ204" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK204" s="2" t="n"/>
+      <c r="AK204" s="3" t="n">
+        <v>-55022.80677563608</v>
+      </c>
       <c r="AL204" s="2" t="n"/>
     </row>
     <row r="205">
@@ -40515,42 +40561,58 @@
         <v>0.01896626502275467</v>
       </c>
       <c r="P206" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q206" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R206" s="2" t="n"/>
-      <c r="S206" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T206" s="2" t="n"/>
-      <c r="U206" s="2" t="n"/>
-      <c r="V206" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q206" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R206" s="3" t="n">
+        <v>-55043.02204937777</v>
+      </c>
+      <c r="S206" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T206" s="3" t="n">
+        <v>12.68671330368252</v>
+      </c>
+      <c r="U206" s="3" t="n">
+        <v>12.68671330368252</v>
+      </c>
+      <c r="V206" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W206" s="2" t="n"/>
       <c r="X206" s="2" t="n"/>
-      <c r="Y206" s="2" t="n"/>
+      <c r="Y206" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z206" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA206" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB206" s="2" t="n"/>
-      <c r="AC206" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD206" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA206" s="2" t="inlineStr"/>
+      <c r="AB206" s="3" t="n">
+        <v>-55030.33533607409</v>
+      </c>
+      <c r="AC206" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD206" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_c285539322fa/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE206" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_c285539322fa/neu/result.json</t>
@@ -40577,7 +40639,9 @@
       <c r="AJ206" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK206" s="2" t="n"/>
+      <c r="AK206" s="3" t="n">
+        <v>-55030.33533607409</v>
+      </c>
       <c r="AL206" s="2" t="n"/>
     </row>
     <row r="207">
@@ -40641,42 +40705,58 @@
         <v>0.01871072314679623</v>
       </c>
       <c r="P207" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q207" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R207" s="2" t="n"/>
-      <c r="S207" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T207" s="2" t="n"/>
-      <c r="U207" s="2" t="n"/>
-      <c r="V207" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q207" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R207" s="3" t="n">
+        <v>-55035.29691748785</v>
+      </c>
+      <c r="S207" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T207" s="3" t="n">
+        <v>12.80489964671403</v>
+      </c>
+      <c r="U207" s="3" t="n">
+        <v>12.80489964671403</v>
+      </c>
+      <c r="V207" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W207" s="2" t="n"/>
       <c r="X207" s="2" t="n"/>
-      <c r="Y207" s="2" t="n"/>
+      <c r="Y207" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z207" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA207" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB207" s="2" t="n"/>
-      <c r="AC207" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD207" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA207" s="2" t="inlineStr"/>
+      <c r="AB207" s="3" t="n">
+        <v>-55022.49201784114</v>
+      </c>
+      <c r="AC207" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD207" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_4602f4a856c7/ox2/result.json</t>
+        </is>
+      </c>
       <c r="AE207" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_4602f4a856c7/ox2/result.json</t>
@@ -40703,7 +40783,9 @@
       <c r="AJ207" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK207" s="2" t="n"/>
+      <c r="AK207" s="3" t="n">
+        <v>-55022.49201784114</v>
+      </c>
       <c r="AL207" s="2" t="n"/>
     </row>
     <row r="208">
@@ -41619,42 +41701,58 @@
         <v>0.01955554820597172</v>
       </c>
       <c r="P214" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q214" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R214" s="2" t="n"/>
-      <c r="S214" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T214" s="2" t="n"/>
-      <c r="U214" s="2" t="n"/>
-      <c r="V214" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q214" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R214" s="3" t="n">
+        <v>-55039.33085085831</v>
+      </c>
+      <c r="S214" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T214" s="3" t="n">
+        <v>12.80321459644746</v>
+      </c>
+      <c r="U214" s="3" t="n">
+        <v>12.80321459644746</v>
+      </c>
+      <c r="V214" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W214" s="2" t="n"/>
       <c r="X214" s="2" t="n"/>
-      <c r="Y214" s="2" t="n"/>
+      <c r="Y214" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z214" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA214" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB214" s="2" t="n"/>
-      <c r="AC214" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD214" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA214" s="2" t="inlineStr"/>
+      <c r="AB214" s="3" t="n">
+        <v>-55026.52763626187</v>
+      </c>
+      <c r="AC214" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD214" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_c88a8d5645d4/ox1/result.json</t>
+        </is>
+      </c>
       <c r="AE214" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_c88a8d5645d4/ox1/result.json</t>
@@ -41679,7 +41777,9 @@
       <c r="AJ214" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK214" s="2" t="n"/>
+      <c r="AK214" s="3" t="n">
+        <v>-55026.52763626187</v>
+      </c>
       <c r="AL214" s="2" t="n"/>
     </row>
     <row r="215">
@@ -41887,14 +41987,16 @@
         <v>0.01989250630140305</v>
       </c>
       <c r="P216" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q216" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R216" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q216" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R216" s="3" t="n">
+        <v>-55035.11388418833</v>
+      </c>
       <c r="S216" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -41902,10 +42004,18 @@
       </c>
       <c r="T216" s="2" t="n"/>
       <c r="U216" s="2" t="n"/>
-      <c r="V216" s="2" t="n"/>
+      <c r="V216" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W216" s="2" t="n"/>
       <c r="X216" s="2" t="n"/>
-      <c r="Y216" s="2" t="n"/>
+      <c r="Y216" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z216" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -41913,7 +42023,7 @@
       </c>
       <c r="AA216" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB216" s="2" t="n"/>
@@ -41922,7 +42032,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD216" s="2" t="n"/>
+      <c r="AD216" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_693080e8c287/ox2/result.json</t>
+        </is>
+      </c>
       <c r="AE216" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_693080e8c287/ox2/result.json</t>
@@ -42013,14 +42127,16 @@
         <v>0.01811725646257401</v>
       </c>
       <c r="P217" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q217" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R217" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q217" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R217" s="3" t="n">
+        <v>-55039.04883038579</v>
+      </c>
       <c r="S217" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -42028,10 +42144,18 @@
       </c>
       <c r="T217" s="2" t="n"/>
       <c r="U217" s="2" t="n"/>
-      <c r="V217" s="2" t="n"/>
+      <c r="V217" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W217" s="2" t="n"/>
       <c r="X217" s="2" t="n"/>
-      <c r="Y217" s="2" t="n"/>
+      <c r="Y217" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z217" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -42039,7 +42163,7 @@
       </c>
       <c r="AA217" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB217" s="2" t="n"/>
@@ -42048,7 +42172,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD217" s="2" t="n"/>
+      <c r="AD217" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_693080e8c287/ox1/result.json</t>
+        </is>
+      </c>
       <c r="AE217" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_693080e8c287/ox1/result.json</t>
@@ -42137,14 +42265,16 @@
         <v>0.01916824840009212</v>
       </c>
       <c r="P218" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q218" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R218" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q218" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R218" s="3" t="n">
+        <v>-55042.43611432912</v>
+      </c>
       <c r="S218" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -42152,10 +42282,18 @@
       </c>
       <c r="T218" s="2" t="n"/>
       <c r="U218" s="2" t="n"/>
-      <c r="V218" s="2" t="n"/>
+      <c r="V218" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W218" s="2" t="n"/>
       <c r="X218" s="2" t="n"/>
-      <c r="Y218" s="2" t="n"/>
+      <c r="Y218" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z218" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -42163,7 +42301,7 @@
       </c>
       <c r="AA218" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB218" s="2" t="n"/>
@@ -42172,7 +42310,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD218" s="2" t="n"/>
+      <c r="AD218" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_693080e8c287/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE218" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_693080e8c287/neu/result.json</t>
@@ -42527,14 +42669,16 @@
         <v>0.018941730260849</v>
       </c>
       <c r="P221" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q221" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R221" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q221" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R221" s="3" t="n">
+        <v>-42701.91452567933</v>
+      </c>
       <c r="S221" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -42542,10 +42686,18 @@
       </c>
       <c r="T221" s="2" t="n"/>
       <c r="U221" s="2" t="n"/>
-      <c r="V221" s="2" t="n"/>
+      <c r="V221" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W221" s="2" t="n"/>
       <c r="X221" s="2" t="n"/>
-      <c r="Y221" s="2" t="n"/>
+      <c r="Y221" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z221" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -42553,7 +42705,7 @@
       </c>
       <c r="AA221" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB221" s="2" t="n"/>
@@ -42562,7 +42714,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD221" s="2" t="n"/>
+      <c r="AD221" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_9992bd3479e1/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE221" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_9992bd3479e1/neu/result.json</t>
@@ -54015,13 +54171,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I132" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J132" s="2" t="n"/>
-      <c r="K132" s="2" t="n"/>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J132" s="3" t="n">
+        <v>3.895</v>
+      </c>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L132" s="2" t="n"/>
       <c r="M132" s="2" t="n"/>
       <c r="N132" s="2" t="n"/>
@@ -54083,13 +54245,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I133" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J133" s="2" t="n"/>
-      <c r="K133" s="2" t="n"/>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J133" s="3" t="n">
+        <v>3.379</v>
+      </c>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L133" s="2" t="n"/>
       <c r="M133" s="2" t="n"/>
       <c r="N133" s="2" t="n"/>
@@ -54151,13 +54319,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I134" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J134" s="2" t="n"/>
-      <c r="K134" s="2" t="n"/>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J134" s="3" t="n">
+        <v>3.926</v>
+      </c>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L134" s="2" t="n"/>
       <c r="M134" s="2" t="n"/>
       <c r="N134" s="2" t="n"/>
@@ -54219,13 +54393,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I135" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J135" s="2" t="n"/>
-      <c r="K135" s="2" t="n"/>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J135" s="3" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L135" s="2" t="n"/>
       <c r="M135" s="2" t="n"/>
       <c r="N135" s="2" t="n"/>
@@ -54423,13 +54603,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I138" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J138" s="2" t="n"/>
-      <c r="K138" s="2" t="n"/>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J138" s="3" t="n">
+        <v>3.967</v>
+      </c>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L138" s="2" t="n"/>
       <c r="M138" s="2" t="n"/>
       <c r="N138" s="2" t="n"/>
@@ -54707,19 +54893,27 @@
       <c r="F142" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G142" s="2" t="n"/>
-      <c r="H142" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I142" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J142" s="2" t="n"/>
-      <c r="K142" s="2" t="n"/>
+      <c r="G142" s="3" t="n">
+        <v>-0.3325872724744841</v>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J142" s="3" t="n">
+        <v>3.935</v>
+      </c>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L142" s="2" t="n"/>
       <c r="M142" s="2" t="n"/>
       <c r="N142" s="2" t="n"/>
@@ -54746,7 +54940,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="T142" s="2" t="n"/>
+      <c r="T142" s="3" t="n">
+        <v>-0.3325872724744841</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -54775,19 +54971,27 @@
       <c r="F143" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G143" s="2" t="n"/>
-      <c r="H143" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I143" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J143" s="2" t="n"/>
-      <c r="K143" s="2" t="n"/>
+      <c r="G143" s="3" t="n">
+        <v>-0.989067565446021</v>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J143" s="3" t="n">
+        <v>3.348</v>
+      </c>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L143" s="2" t="n"/>
       <c r="M143" s="2" t="n"/>
       <c r="N143" s="2" t="n"/>
@@ -54814,7 +55018,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="T143" s="2" t="n"/>
+      <c r="T143" s="3" t="n">
+        <v>-0.989067565446021</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -54849,13 +55055,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I144" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J144" s="2" t="n"/>
-      <c r="K144" s="2" t="n"/>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J144" s="3" t="n">
+        <v>3.935</v>
+      </c>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L144" s="2" t="n"/>
       <c r="M144" s="2" t="n"/>
       <c r="N144" s="2" t="n"/>
@@ -54917,13 +55129,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I145" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J145" s="2" t="n"/>
-      <c r="K145" s="2" t="n"/>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J145" s="3" t="n">
+        <v>3.387</v>
+      </c>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L145" s="2" t="n"/>
       <c r="M145" s="2" t="n"/>
       <c r="N145" s="2" t="n"/>
@@ -62250,10 +62468,10 @@
         <v>3</v>
       </c>
       <c r="AB29" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC29" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD29" s="2" t="n">
         <v>0</v>
@@ -62302,7 +62520,7 @@
       </c>
       <c r="AU29" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV29" s="2" t="n"/>
@@ -62339,7 +62557,7 @@
       <c r="BK29" s="2" t="n"/>
       <c r="BL29" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 2 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 1 resource-deferred; field-specific QC separate</t>
+          <t>0/3 surface records verified; 2 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM29" s="2" t="b">
@@ -62451,10 +62669,10 @@
         <v>3</v>
       </c>
       <c r="AB30" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD30" s="2" t="n">
         <v>0</v>
@@ -62503,7 +62721,7 @@
       </c>
       <c r="AU30" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV30" s="2" t="n"/>
@@ -62540,7 +62758,7 @@
       <c r="BK30" s="2" t="n"/>
       <c r="BL30" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 3 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>0/3 surface records verified; 2 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM30" s="2" t="b">
@@ -62567,7 +62785,7 @@
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>partial native solution states; remaining states pending</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -62652,16 +62870,16 @@
         <v>3</v>
       </c>
       <c r="AB31" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC31" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD31" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE31" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF31" s="4" t="inlineStr">
         <is>
@@ -62714,7 +62932,7 @@
       <c r="AZ31" s="2" t="n"/>
       <c r="BA31" s="2" t="n"/>
       <c r="BB31" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BC31" s="2" t="inlineStr">
         <is>
@@ -62741,7 +62959,7 @@
       <c r="BK31" s="2" t="n"/>
       <c r="BL31" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 2 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 1 resource-deferred; field-specific QC separate</t>
+          <t>2/3 surface records verified; 0 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM31" s="2" t="b">
@@ -62853,16 +63071,16 @@
         <v>3</v>
       </c>
       <c r="AB32" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC32" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD32" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="AC32" s="2" t="n">
+      <c r="AE32" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="AD32" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE32" s="2" t="n">
-        <v>1</v>
       </c>
       <c r="AF32" s="4" t="inlineStr">
         <is>
@@ -62905,7 +63123,7 @@
       </c>
       <c r="AU32" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV32" s="2" t="n"/>
@@ -62915,7 +63133,7 @@
       <c r="AZ32" s="2" t="n"/>
       <c r="BA32" s="2" t="n"/>
       <c r="BB32" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BC32" s="2" t="inlineStr">
         <is>
@@ -62942,7 +63160,7 @@
       <c r="BK32" s="2" t="n"/>
       <c r="BL32" s="2" t="inlineStr">
         <is>
-          <t>1/3 surface records verified; 1 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>2/3 surface records verified; 1 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM32" s="2" t="b">
@@ -63143,7 +63361,7 @@
       <c r="BK33" s="2" t="n"/>
       <c r="BL33" s="2" t="inlineStr">
         <is>
-          <t>2/3 surface records verified; 0 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>2/3 surface records verified; 1 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM33" s="2" t="b">
@@ -63170,7 +63388,7 @@
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>partial native solution states; remaining states pending</t>
+          <t>native solution states complete</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -63255,29 +63473,37 @@
         <v>3</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD34" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE34" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF34" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AG34" s="2" t="n"/>
-      <c r="AH34" s="2" t="n"/>
-      <c r="AI34" s="2" t="n"/>
-      <c r="AJ34" s="2" t="n"/>
-      <c r="AK34" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+        <v>3</v>
+      </c>
+      <c r="AF34" s="2" t="inlineStr">
+        <is>
+          <t>verified native calculation</t>
+        </is>
+      </c>
+      <c r="AG34" s="3" t="n">
+        <v>-0.3325872724744841</v>
+      </c>
+      <c r="AH34" s="3" t="n">
+        <v>-0.989067565446021</v>
+      </c>
+      <c r="AI34" s="3" t="n">
+        <v>0.6564802929788129</v>
+      </c>
+      <c r="AJ34" s="3" t="n">
+        <v>63.34071909829567</v>
+      </c>
+      <c r="AK34" s="2" t="inlineStr">
+        <is>
+          <t>native thermodynamic calculation; decomposition untested</t>
         </is>
       </c>
       <c r="AL34" s="4" t="inlineStr">
@@ -63289,10 +63515,12 @@
       <c r="AN34" s="2" t="n"/>
       <c r="AO34" s="2" t="inlineStr">
         <is>
-          <t>pending electrolyte-window/integrity QC</t>
-        </is>
-      </c>
-      <c r="AP34" s="2" t="n"/>
+          <t>computed native-window/integrity bookkeeping; kinetic QC separate</t>
+        </is>
+      </c>
+      <c r="AP34" s="3" t="n">
+        <v>90.76202409952268</v>
+      </c>
       <c r="AQ34" s="2" t="b">
         <v>0</v>
       </c>
@@ -63307,7 +63535,7 @@
       </c>
       <c r="AU34" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV34" s="2" t="n"/>
@@ -63317,7 +63545,7 @@
       <c r="AZ34" s="2" t="n"/>
       <c r="BA34" s="2" t="n"/>
       <c r="BB34" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC34" s="2" t="inlineStr">
         <is>
@@ -63329,8 +63557,12 @@
           <t>ox2:UMA_large_gap_preliminary; ox1:standard_doublet_model; neu:UMA_large_gap_preliminary</t>
         </is>
       </c>
-      <c r="BE34" s="2" t="n"/>
-      <c r="BF34" s="2" t="n"/>
+      <c r="BE34" s="3" t="n">
+        <v>-0.3325872724744841</v>
+      </c>
+      <c r="BF34" s="3" t="n">
+        <v>-0.989067565446021</v>
+      </c>
       <c r="BG34" s="2" t="b">
         <v>1</v>
       </c>
@@ -63341,10 +63573,12 @@
       </c>
       <c r="BI34" s="2" t="n"/>
       <c r="BJ34" s="2" t="n"/>
-      <c r="BK34" s="2" t="n"/>
+      <c r="BK34" s="3" t="n">
+        <v>90.76202409952268</v>
+      </c>
       <c r="BL34" s="2" t="inlineStr">
         <is>
-          <t>2/3 surface records verified; 0 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>3/3 surface records verified; 0 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM34" s="2" t="b">
@@ -63371,7 +63605,7 @@
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>active SP records present; native validation pending</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -63456,10 +63690,10 @@
         <v>3</v>
       </c>
       <c r="AB35" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC35" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD35" s="2" t="n">
         <v>0</v>
@@ -63508,7 +63742,7 @@
       </c>
       <c r="AU35" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV35" s="2" t="n"/>
@@ -63545,7 +63779,7 @@
       <c r="BK35" s="2" t="n"/>
       <c r="BL35" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 3 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>0/3 surface records verified; 3 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM35" s="2" t="b">
@@ -63657,10 +63891,10 @@
         <v>3</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD36" s="2" t="n">
         <v>0</v>
@@ -63746,7 +63980,7 @@
       <c r="BK36" s="2" t="n"/>
       <c r="BL36" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 2 producer reports in progress; 0 queued/unresolved; 1 resource-deferred; field-specific QC separate</t>
+          <t>0/3 surface records verified; 2 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM36" s="2" t="b">
@@ -63947,7 +64181,7 @@
       <c r="BK37" s="2" t="n"/>
       <c r="BL37" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 2 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 1 resource-deferred; field-specific QC separate</t>
+          <t>0/3 surface records verified; 0 failed/preserved; 3 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM37" s="2" t="b">
@@ -65629,7 +65863,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-19T12:22:05.478576-05:00</t>
+          <t>2026-10-19T13:27:36.549685-05:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Visualize parent validation and candidate selection for post-grafting research
</commit_message>
<xml_diff>
--- a/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
+++ b/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
@@ -40025,13 +40025,17 @@
       <c r="R202" s="3" t="n">
         <v>-44774.14750819249</v>
       </c>
-      <c r="S202" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T202" s="2" t="n"/>
-      <c r="U202" s="2" t="n"/>
+      <c r="S202" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T202" s="3" t="n">
+        <v>12.13570876705565</v>
+      </c>
+      <c r="U202" s="3" t="n">
+        <v>12.13570876705565</v>
+      </c>
       <c r="V202" s="2" t="inlineStr">
         <is>
           <t>not_selected</t>
@@ -40046,18 +40050,16 @@
       </c>
       <c r="Z202" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA202" s="2" t="inlineStr">
-        <is>
-          <t>missing_validated_native_thermal</t>
-        </is>
-      </c>
-      <c r="AB202" s="2" t="n"/>
-      <c r="AC202" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA202" s="2" t="inlineStr"/>
+      <c r="AB202" s="3" t="n">
+        <v>-44762.01179942544</v>
+      </c>
+      <c r="AC202" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
         </is>
       </c>
       <c r="AD202" s="2" t="inlineStr">
@@ -40089,7 +40091,9 @@
       <c r="AJ202" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK202" s="2" t="n"/>
+      <c r="AK202" s="3" t="n">
+        <v>-44762.01179942544</v>
+      </c>
       <c r="AL202" s="2" t="n"/>
     </row>
     <row r="203">
@@ -40437,42 +40441,58 @@
         <v>0.01956345699727535</v>
       </c>
       <c r="P205" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q205" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R205" s="2" t="n"/>
-      <c r="S205" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T205" s="2" t="n"/>
-      <c r="U205" s="2" t="n"/>
-      <c r="V205" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q205" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R205" s="3" t="n">
+        <v>-55039.58680064894</v>
+      </c>
+      <c r="S205" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T205" s="3" t="n">
+        <v>12.74266549154393</v>
+      </c>
+      <c r="U205" s="3" t="n">
+        <v>12.74266549154393</v>
+      </c>
+      <c r="V205" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W205" s="2" t="n"/>
       <c r="X205" s="2" t="n"/>
-      <c r="Y205" s="2" t="n"/>
+      <c r="Y205" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z205" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA205" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB205" s="2" t="n"/>
-      <c r="AC205" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD205" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA205" s="2" t="inlineStr"/>
+      <c r="AB205" s="3" t="n">
+        <v>-55026.84413515739</v>
+      </c>
+      <c r="AC205" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD205" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_c285539322fa/ox1/result.json</t>
+        </is>
+      </c>
       <c r="AE205" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_c285539322fa/ox1/result.json</t>
@@ -40497,7 +40517,9 @@
       <c r="AJ205" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK205" s="2" t="n"/>
+      <c r="AK205" s="3" t="n">
+        <v>-55026.84413515739</v>
+      </c>
       <c r="AL205" s="2" t="n"/>
     </row>
     <row r="206">
@@ -42545,14 +42567,16 @@
         <v>0.01773704402148724</v>
       </c>
       <c r="P220" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q220" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R220" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q220" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R220" s="3" t="n">
+        <v>-42698.64117892488</v>
+      </c>
       <c r="S220" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -42560,10 +42584,18 @@
       </c>
       <c r="T220" s="2" t="n"/>
       <c r="U220" s="2" t="n"/>
-      <c r="V220" s="2" t="n"/>
+      <c r="V220" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W220" s="2" t="n"/>
       <c r="X220" s="2" t="n"/>
-      <c r="Y220" s="2" t="n"/>
+      <c r="Y220" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z220" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -42571,7 +42603,7 @@
       </c>
       <c r="AA220" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB220" s="2" t="n"/>
@@ -42580,7 +42612,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD220" s="2" t="n"/>
+      <c r="AD220" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_9992bd3479e1/ox1/result.json</t>
+        </is>
+      </c>
       <c r="AE220" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_9992bd3479e1/ox1/result.json</t>
@@ -42809,14 +42845,16 @@
         <v>0.01951351948082447</v>
       </c>
       <c r="P222" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q222" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R222" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q222" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R222" s="3" t="n">
+        <v>-42694.73044996935</v>
+      </c>
       <c r="S222" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -42824,10 +42862,18 @@
       </c>
       <c r="T222" s="2" t="n"/>
       <c r="U222" s="2" t="n"/>
-      <c r="V222" s="2" t="n"/>
+      <c r="V222" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W222" s="2" t="n"/>
       <c r="X222" s="2" t="n"/>
-      <c r="Y222" s="2" t="n"/>
+      <c r="Y222" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z222" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -42835,7 +42881,7 @@
       </c>
       <c r="AA222" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB222" s="2" t="n"/>
@@ -42844,7 +42890,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD222" s="2" t="n"/>
+      <c r="AD222" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_6f1ff24b8d40/ox2/result.json</t>
+        </is>
+      </c>
       <c r="AE222" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_6f1ff24b8d40/ox2/result.json</t>
@@ -42935,14 +42985,16 @@
         <v>0.01917439512908459</v>
       </c>
       <c r="P223" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q223" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R223" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q223" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R223" s="3" t="n">
+        <v>-42698.59935644037</v>
+      </c>
       <c r="S223" s="4" t="inlineStr">
         <is>
           <t>pending</t>
@@ -42950,10 +43002,18 @@
       </c>
       <c r="T223" s="2" t="n"/>
       <c r="U223" s="2" t="n"/>
-      <c r="V223" s="2" t="n"/>
+      <c r="V223" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W223" s="2" t="n"/>
       <c r="X223" s="2" t="n"/>
-      <c r="Y223" s="2" t="n"/>
+      <c r="Y223" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z223" s="2" t="inlineStr">
         <is>
           <t>INCOMPLETE</t>
@@ -42961,7 +43021,7 @@
       </c>
       <c r="AA223" s="2" t="inlineStr">
         <is>
-          <t>missing_geometry_or_result</t>
+          <t>missing_validated_native_thermal</t>
         </is>
       </c>
       <c r="AB223" s="2" t="n"/>
@@ -42970,7 +43030,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="AD223" s="2" t="n"/>
+      <c r="AD223" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_6f1ff24b8d40/ox1/result.json</t>
+        </is>
+      </c>
       <c r="AE223" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_6f1ff24b8d40/ox1/result.json</t>
@@ -43059,42 +43123,58 @@
         <v>0.01843639276921749</v>
       </c>
       <c r="P224" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q224" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R224" s="2" t="n"/>
-      <c r="S224" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="T224" s="2" t="n"/>
-      <c r="U224" s="2" t="n"/>
-      <c r="V224" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="Q224" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="R224" s="3" t="n">
+        <v>-42701.86574662838</v>
+      </c>
+      <c r="S224" s="2" t="inlineStr">
+        <is>
+          <t>addressed QC passed</t>
+        </is>
+      </c>
+      <c r="T224" s="3" t="n">
+        <v>11.74983516977084</v>
+      </c>
+      <c r="U224" s="3" t="n">
+        <v>11.74983516977084</v>
+      </c>
+      <c r="V224" s="2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
       <c r="W224" s="2" t="n"/>
       <c r="X224" s="2" t="n"/>
-      <c r="Y224" s="2" t="n"/>
+      <c r="Y224" s="2" t="inlineStr">
+        <is>
+          <t>native_solution_dft_qrrho_spin</t>
+        </is>
+      </c>
       <c r="Z224" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="AA224" s="2" t="inlineStr">
-        <is>
-          <t>missing_geometry_or_result</t>
-        </is>
-      </c>
-      <c r="AB224" s="2" t="n"/>
-      <c r="AC224" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AD224" s="2" t="n"/>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="AA224" s="2" t="inlineStr"/>
+      <c r="AB224" s="3" t="n">
+        <v>-42690.11591145861</v>
+      </c>
+      <c r="AC224" s="2" t="inlineStr">
+        <is>
+          <t>verified calculation</t>
+        </is>
+      </c>
+      <c r="AD224" s="2" t="inlineStr">
+        <is>
+          <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/dft/study_aryl_6f1ff24b8d40/neu/result.json</t>
+        </is>
+      </c>
       <c r="AE224" s="2" t="inlineStr">
         <is>
           <t>/nfs/lambda_stor_01/homes/rzhu/0_redox/calcs/uma/study_aryl_6f1ff24b8d40/neu/result.json</t>
@@ -43121,7 +43201,9 @@
       <c r="AJ224" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AK224" s="2" t="n"/>
+      <c r="AK224" s="3" t="n">
+        <v>-42690.11591145861</v>
+      </c>
       <c r="AL224" s="2" t="n"/>
     </row>
     <row r="225">
@@ -54461,19 +54543,27 @@
       <c r="F136" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G136" s="2" t="n"/>
-      <c r="H136" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I136" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J136" s="2" t="n"/>
-      <c r="K136" s="2" t="n"/>
+      <c r="G136" s="3" t="n">
+        <v>-0.3418363802848035</v>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J136" s="3" t="n">
+        <v>3.947</v>
+      </c>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L136" s="2" t="n"/>
       <c r="M136" s="2" t="n"/>
       <c r="N136" s="2" t="n"/>
@@ -54500,7 +54590,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="T136" s="2" t="n"/>
+      <c r="T136" s="3" t="n">
+        <v>-0.3418363802848035</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -54529,19 +54621,27 @@
       <c r="F137" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G137" s="2" t="n"/>
-      <c r="H137" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I137" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J137" s="2" t="n"/>
-      <c r="K137" s="2" t="n"/>
+      <c r="G137" s="3" t="n">
+        <v>-0.8879949848997057</v>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>native calculated/QC passed</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J137" s="3" t="n">
+        <v>3.435</v>
+      </c>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L137" s="2" t="n"/>
       <c r="M137" s="2" t="n"/>
       <c r="N137" s="2" t="n"/>
@@ -54568,7 +54668,9 @@
           <t>admissible under stated spin evidence</t>
         </is>
       </c>
-      <c r="T137" s="2" t="n"/>
+      <c r="T137" s="3" t="n">
+        <v>-0.8879949848997057</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -55203,13 +55305,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I146" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J146" s="2" t="n"/>
-      <c r="K146" s="2" t="n"/>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J146" s="3" t="n">
+        <v>3.847</v>
+      </c>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L146" s="2" t="n"/>
       <c r="M146" s="2" t="n"/>
       <c r="N146" s="2" t="n"/>
@@ -55271,13 +55379,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I147" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J147" s="2" t="n"/>
-      <c r="K147" s="2" t="n"/>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J147" s="3" t="n">
+        <v>3.273</v>
+      </c>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L147" s="2" t="n"/>
       <c r="M147" s="2" t="n"/>
       <c r="N147" s="2" t="n"/>
@@ -55339,13 +55453,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I148" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J148" s="2" t="n"/>
-      <c r="K148" s="2" t="n"/>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J148" s="3" t="n">
+        <v>3.869</v>
+      </c>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L148" s="2" t="n"/>
       <c r="M148" s="2" t="n"/>
       <c r="N148" s="2" t="n"/>
@@ -55407,13 +55527,19 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="I149" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="J149" s="2" t="n"/>
-      <c r="K149" s="2" t="n"/>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>intact_bound</t>
+        </is>
+      </c>
+      <c r="J149" s="3" t="n">
+        <v>3.266</v>
+      </c>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
       <c r="L149" s="2" t="n"/>
       <c r="M149" s="2" t="n"/>
       <c r="N149" s="2" t="n"/>
@@ -62557,7 +62683,7 @@
       <c r="BK29" s="2" t="n"/>
       <c r="BL29" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 2 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>0/3 surface records verified; 3 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM29" s="2" t="b">
@@ -62584,7 +62710,7 @@
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>active SP records present; native validation pending</t>
+          <t>partial native solution states; remaining states pending</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -62675,10 +62801,10 @@
         <v>3</v>
       </c>
       <c r="AD30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF30" s="4" t="inlineStr">
         <is>
@@ -62731,7 +62857,7 @@
       <c r="AZ30" s="2" t="n"/>
       <c r="BA30" s="2" t="n"/>
       <c r="BB30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC30" s="2" t="inlineStr">
         <is>
@@ -62758,7 +62884,7 @@
       <c r="BK30" s="2" t="n"/>
       <c r="BL30" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 2 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>1/3 surface records verified; 2 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM30" s="2" t="b">
@@ -62785,7 +62911,7 @@
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>partial native solution states; remaining states pending</t>
+          <t>native solution states complete</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -62870,29 +62996,37 @@
         <v>3</v>
       </c>
       <c r="AB31" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC31" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD31" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE31" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF31" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="AG31" s="2" t="n"/>
-      <c r="AH31" s="2" t="n"/>
-      <c r="AI31" s="2" t="n"/>
-      <c r="AJ31" s="2" t="n"/>
-      <c r="AK31" s="4" t="inlineStr">
-        <is>
-          <t>pending</t>
+        <v>3</v>
+      </c>
+      <c r="AF31" s="2" t="inlineStr">
+        <is>
+          <t>verified native calculation</t>
+        </is>
+      </c>
+      <c r="AG31" s="3" t="n">
+        <v>-0.3418363802848035</v>
+      </c>
+      <c r="AH31" s="3" t="n">
+        <v>-0.8879949848997057</v>
+      </c>
+      <c r="AI31" s="3" t="n">
+        <v>0.5461586046149023</v>
+      </c>
+      <c r="AJ31" s="3" t="n">
+        <v>52.69629435646461</v>
+      </c>
+      <c r="AK31" s="2" t="inlineStr">
+        <is>
+          <t>native thermodynamic calculation; decomposition untested</t>
         </is>
       </c>
       <c r="AL31" s="4" t="inlineStr">
@@ -62904,10 +63038,12 @@
       <c r="AN31" s="2" t="n"/>
       <c r="AO31" s="2" t="inlineStr">
         <is>
-          <t>pending electrolyte-window/integrity QC</t>
-        </is>
-      </c>
-      <c r="AP31" s="2" t="n"/>
+          <t>computed native-window/integrity bookkeeping; kinetic QC separate</t>
+        </is>
+      </c>
+      <c r="AP31" s="3" t="n">
+        <v>90.76202409952268</v>
+      </c>
       <c r="AQ31" s="2" t="b">
         <v>0</v>
       </c>
@@ -62922,7 +63058,7 @@
       </c>
       <c r="AU31" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV31" s="2" t="n"/>
@@ -62932,7 +63068,7 @@
       <c r="AZ31" s="2" t="n"/>
       <c r="BA31" s="2" t="n"/>
       <c r="BB31" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC31" s="2" t="inlineStr">
         <is>
@@ -62944,8 +63080,12 @@
           <t>ox2:UMA_large_gap_preliminary; ox1:standard_doublet_model; neu:UMA_large_gap_preliminary</t>
         </is>
       </c>
-      <c r="BE31" s="2" t="n"/>
-      <c r="BF31" s="2" t="n"/>
+      <c r="BE31" s="3" t="n">
+        <v>-0.3418363802848035</v>
+      </c>
+      <c r="BF31" s="3" t="n">
+        <v>-0.8879949848997057</v>
+      </c>
       <c r="BG31" s="2" t="b">
         <v>1</v>
       </c>
@@ -62956,10 +63096,12 @@
       </c>
       <c r="BI31" s="2" t="n"/>
       <c r="BJ31" s="2" t="n"/>
-      <c r="BK31" s="2" t="n"/>
+      <c r="BK31" s="3" t="n">
+        <v>90.76202409952268</v>
+      </c>
       <c r="BL31" s="2" t="inlineStr">
         <is>
-          <t>2/3 surface records verified; 0 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>3/3 surface records verified; 0 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM31" s="2" t="b">
@@ -63891,10 +64033,10 @@
         <v>3</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD36" s="2" t="n">
         <v>0</v>
@@ -63943,7 +64085,7 @@
       </c>
       <c r="AU36" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV36" s="2" t="n"/>
@@ -63980,7 +64122,7 @@
       <c r="BK36" s="2" t="n"/>
       <c r="BL36" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 2 failed/preserved; 1 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>0/3 surface records verified; 3 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM36" s="2" t="b">
@@ -64007,7 +64149,7 @@
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>gas UMA only</t>
+          <t>partial native solution states; remaining states pending</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -64092,16 +64234,16 @@
         <v>3</v>
       </c>
       <c r="AB37" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC37" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD37" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE37" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF37" s="4" t="inlineStr">
         <is>
@@ -64144,7 +64286,7 @@
       </c>
       <c r="AU37" s="2" t="inlineStr">
         <is>
-          <t>remaining DFT geometry records; remaining active SP records; native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
+          <t>native Hessian/derivative and solution-admission QC; matched-reference redox potentials; field-specific integrity/reorganization and window gates</t>
         </is>
       </c>
       <c r="AV37" s="2" t="n"/>
@@ -64154,7 +64296,7 @@
       <c r="AZ37" s="2" t="n"/>
       <c r="BA37" s="2" t="n"/>
       <c r="BB37" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC37" s="2" t="inlineStr">
         <is>
@@ -64181,7 +64323,7 @@
       <c r="BK37" s="2" t="n"/>
       <c r="BL37" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 0 failed/preserved; 3 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>1/3 surface records verified; 2 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
         </is>
       </c>
       <c r="BM37" s="2" t="b">
@@ -65863,7 +66005,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-19T13:27:36.549685-05:00</t>
+          <t>2026-10-19T18:29:30.930801-05:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Require every candidate axis to pass before Pareto selection
Add exact-identity, scope, context and interval-aware admission to the
normal candidate publication workflow. Preserve incomplete evidence as
pending and keep descriptor fronts separate from a material shortlist.

Publish the source-current decision ledger, focused 34-slot expansion
plan and checked figures. No candidate passes all required criteria.
Reconstruct benchmark/candidate evidence without changing their values.

Preserve and verify twelve expanded CPU CREST searches across six
occupancy graphs and two configurations; DFT ensembles remain pending.
Respect large bound CPU allocations and record actual worker ownership.

Validation: 805 full-suite passes, one plotting dependency skip passed
separately, and two subsequent slide-boundary regressions pass.
Independent publication replay checks 879 exact graphs and all source
hashes. Refresh and visually check changed pages of the 71-page deck.
</commit_message>
<xml_diff>
--- a/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
+++ b/results/reviews/2026-10-18/verified_candidates/LATEST_verified_candidates.xlsx
@@ -2443,7 +2443,7 @@
       </c>
       <c r="BL2" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM2" s="2" t="b">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="BL3" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM3" s="2" t="b">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="BL4" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM4" s="2" t="b">
@@ -3130,7 +3130,7 @@
       </c>
       <c r="BL5" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM5" s="2" t="b">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="BL6" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM6" s="2" t="b">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="BL7" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM7" s="2" t="b">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="BL8" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM8" s="2" t="b">
@@ -4034,7 +4034,7 @@
       <c r="BK9" s="2" t="n"/>
       <c r="BL9" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM9" s="2" t="b">
@@ -4263,7 +4263,7 @@
       </c>
       <c r="BL10" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM10" s="2" t="b">
@@ -4476,7 +4476,7 @@
       <c r="BK11" s="2" t="n"/>
       <c r="BL11" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM11" s="2" t="b">
@@ -4693,7 +4693,7 @@
       <c r="BK12" s="2" t="n"/>
       <c r="BL12" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM12" s="2" t="b">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="BL13" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM13" s="2" t="b">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="BL14" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM14" s="2" t="b">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="BL15" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM15" s="2" t="b">
@@ -5609,7 +5609,7 @@
       </c>
       <c r="BL16" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM16" s="2" t="b">
@@ -5838,7 +5838,7 @@
       </c>
       <c r="BL17" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM17" s="2" t="b">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="BL18" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM18" s="2" t="b">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="BL19" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM19" s="2" t="b">
@@ -6525,7 +6525,7 @@
       </c>
       <c r="BL20" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM20" s="2" t="b">
@@ -6742,7 +6742,7 @@
       <c r="BK21" s="2" t="n"/>
       <c r="BL21" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM21" s="2" t="b">
@@ -6971,7 +6971,7 @@
       </c>
       <c r="BL22" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM22" s="2" t="b">
@@ -7200,7 +7200,7 @@
       </c>
       <c r="BL23" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM23" s="2" t="b">
@@ -7429,7 +7429,7 @@
       </c>
       <c r="BL24" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM24" s="2" t="b">
@@ -7658,7 +7658,7 @@
       </c>
       <c r="BL25" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM25" s="2" t="b">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="BL26" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM26" s="2" t="b">
@@ -8100,7 +8100,7 @@
       <c r="BK27" s="2" t="n"/>
       <c r="BL27" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM27" s="2" t="b">
@@ -8329,7 +8329,7 @@
       </c>
       <c r="BL28" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM28" s="2" t="b">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="BL29" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM29" s="2" t="b">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="BL30" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM30" s="2" t="b">
@@ -9016,7 +9016,7 @@
       </c>
       <c r="BL31" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM31" s="2" t="b">
@@ -9245,7 +9245,7 @@
       </c>
       <c r="BL32" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM32" s="2" t="b">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="BL33" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM33" s="2" t="b">
@@ -9703,7 +9703,7 @@
       </c>
       <c r="BL34" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM34" s="2" t="b">
@@ -9932,7 +9932,7 @@
       </c>
       <c r="BL35" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM35" s="2" t="b">
@@ -10161,7 +10161,7 @@
       </c>
       <c r="BL36" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM36" s="2" t="b">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="BL37" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM37" s="2" t="b">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="BL38" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM38" s="2" t="b">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="BL39" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM39" s="2" t="b">
@@ -11065,7 +11065,7 @@
       </c>
       <c r="BL40" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>worker done marker; record QC separate</t>
         </is>
       </c>
       <c r="BM40" s="2" t="b">
@@ -56336,7 +56336,7 @@
       <c r="BK2" s="2" t="n"/>
       <c r="BL2" s="2" t="inlineStr">
         <is>
-          <t>outside current queue</t>
+          <t>terminal failure; partial data preserved</t>
         </is>
       </c>
       <c r="BM2" s="2" t="b">
@@ -62683,7 +62683,7 @@
       <c r="BK29" s="2" t="n"/>
       <c r="BL29" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 3 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>outside current queue</t>
         </is>
       </c>
       <c r="BM29" s="2" t="b">
@@ -62884,7 +62884,7 @@
       <c r="BK30" s="2" t="n"/>
       <c r="BL30" s="2" t="inlineStr">
         <is>
-          <t>1/3 surface records verified; 2 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>outside current queue</t>
         </is>
       </c>
       <c r="BM30" s="2" t="b">
@@ -63101,7 +63101,7 @@
       </c>
       <c r="BL31" s="2" t="inlineStr">
         <is>
-          <t>3/3 surface records verified; 0 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>outside current queue</t>
         </is>
       </c>
       <c r="BM31" s="2" t="b">
@@ -63302,7 +63302,7 @@
       <c r="BK32" s="2" t="n"/>
       <c r="BL32" s="2" t="inlineStr">
         <is>
-          <t>2/3 surface records verified; 1 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>outside current queue</t>
         </is>
       </c>
       <c r="BM32" s="2" t="b">
@@ -63503,7 +63503,7 @@
       <c r="BK33" s="2" t="n"/>
       <c r="BL33" s="2" t="inlineStr">
         <is>
-          <t>2/3 surface records verified; 1 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>outside current queue</t>
         </is>
       </c>
       <c r="BM33" s="2" t="b">
@@ -63720,7 +63720,7 @@
       </c>
       <c r="BL34" s="2" t="inlineStr">
         <is>
-          <t>3/3 surface records verified; 0 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>outside current queue</t>
         </is>
       </c>
       <c r="BM34" s="2" t="b">
@@ -63921,7 +63921,7 @@
       <c r="BK35" s="2" t="n"/>
       <c r="BL35" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 3 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>outside current queue</t>
         </is>
       </c>
       <c r="BM35" s="2" t="b">
@@ -64122,7 +64122,7 @@
       <c r="BK36" s="2" t="n"/>
       <c r="BL36" s="2" t="inlineStr">
         <is>
-          <t>0/3 surface records verified; 3 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>outside current queue</t>
         </is>
       </c>
       <c r="BM36" s="2" t="b">
@@ -64323,7 +64323,7 @@
       <c r="BK37" s="2" t="n"/>
       <c r="BL37" s="2" t="inlineStr">
         <is>
-          <t>1/3 surface records verified; 2 failed/preserved; 0 producer reports in progress; 0 queued/unresolved; 0 resource-deferred; field-specific QC separate</t>
+          <t>outside current queue</t>
         </is>
       </c>
       <c r="BM37" s="2" t="b">
@@ -66005,7 +66005,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-19T18:29:30.930801-05:00</t>
+          <t>2026-10-23T03:26:56.484627-05:00</t>
         </is>
       </c>
     </row>

</xml_diff>